<commit_message>
Sources steps 1 and 2: real pacing guide sources, molly duplicate, unsourced claims
Pacing guide placeholder links replaced with the VCA, AVMA and ACVB pages it
names; molly cost guide duplicate removed; White's tree frog and fire-bellied
toad claims rewritten to their listed sources; guppy health guide swaps
Tankarium for Merck and adds Chervinski 1984 for salt.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SOURCE_OVERLAP.xlsx
+++ b/SOURCE_OVERLAP.xlsx
@@ -38,7 +38,7 @@
       <sz val="14"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -65,6 +65,11 @@
         <fgColor rgb="00D9D9D9"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -78,7 +83,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -98,6 +103,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -658,7 +666,6 @@
         <v>4</v>
       </c>
     </row>
-    <row r="21"/>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
@@ -9230,7 +9237,7 @@
       </c>
       <c r="K211" s="5" t="inlineStr">
         <is>
-          <t>FIX_PLAN: the 50 to 68F comfort band; Merck (65 to 80F) and PetMD (55 to 70F) run warmer. Settle one band with sources.</t>
+          <t>FIX_PLAN: the 50 to 68F comfort band; Merck (65 to 80F) and PetMD (55 to 70F) run warmer. Settle one band with sources. 2026-10-06: sources disagree. VCA (listed on the heat stress guide) 50 to 68F; PetMD 55 to 70F, never over 80; LafeberVet 59 to 70F; Merck 65 to 80F adapted range. The setup guide lists PetMD, LafeberVet and Merck but not VCA. Owner call.</t>
         </is>
       </c>
     </row>
@@ -13019,14 +13026,14 @@
       <c r="G307" s="5" t="inlineStr"/>
       <c r="H307" s="5" t="inlineStr"/>
       <c r="I307" s="5" t="inlineStr"/>
-      <c r="J307" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J307" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K307" s="5" t="inlineStr">
         <is>
-          <t>FIX_PLAN: no listed source for the skin toxin harming tankmates of other species, or the small net as a handling option.</t>
+          <t>FIX_PLAN: no listed source for the skin toxin harming tankmates of other species, or the small net as a handling option. 2026-10-06: tankmate line tied to Smithsonian; net option removed.</t>
         </is>
       </c>
     </row>
@@ -16905,14 +16912,14 @@
       <c r="G405" s="5" t="inlineStr"/>
       <c r="H405" s="5" t="inlineStr"/>
       <c r="I405" s="5" t="inlineStr"/>
-      <c r="J405" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J405" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K405" s="5" t="inlineStr">
         <is>
-          <t>FIX_PLAN: Tankarium is still listed and says guppies are not salt tolerant, against the page. Swap it for Chervinski 1984 (Journal of Fish Biology) or trim it.</t>
+          <t>FIX_PLAN: Tankarium is still listed and says guppies are not salt tolerant, against the page. Swap it for Chervinski 1984 (Journal of Fish Biology) or trim it. 2026-10-06: Tankarium replaced by Merck; Chervinski 1984 added. 4 sources.</t>
         </is>
       </c>
     </row>
@@ -21640,12 +21647,16 @@
           <t>Delete the duplicate entry. Combine aquariumcoop.com into one entry linking the site and naming the pages: Molly Fish Care Guide; Care Guide for Mollies.</t>
         </is>
       </c>
-      <c r="J522" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
-        </is>
-      </c>
-      <c r="K522" s="5" t="inlineStr"/>
+      <c r="J522" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K522" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: duplicate Aquarium Co-Op entry removed; 3 sources.</t>
+        </is>
+      </c>
     </row>
     <row r="523">
       <c r="A523" s="5" t="inlineStr">
@@ -30970,12 +30981,16 @@
           <t>Replace each placeholder with the real page it names, or remove it; never leave a link to the site itself.</t>
         </is>
       </c>
-      <c r="J756" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
-        </is>
-      </c>
-      <c r="K756" s="5" t="inlineStr"/>
+      <c r="J756" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K756" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: placeholders replaced with the real pages: VCA (stressed dog signs, fears and anxiety, kitten hiding) in one entry, AVMA JAVMA News Back-to-Work Pet Anxiety, and ACVB What Is a Veterinary Behaviorist. Coal Creek dropped (no page found that the article needs). Cat stress signs reworded to what VCA says: dilated pupils, flat ears, hunched posture.</t>
+        </is>
+      </c>
     </row>
     <row r="757">
       <c r="A757" s="5" t="inlineStr">
@@ -31110,14 +31125,14 @@
       <c r="G760" s="5" t="inlineStr"/>
       <c r="H760" s="5" t="inlineStr"/>
       <c r="I760" s="5" t="inlineStr"/>
-      <c r="J760" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J760" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K760" s="5" t="inlineStr">
         <is>
-          <t>FIX_PLAN: no listed source for 5 to 15 minute sessions about twice a week, larger and hardier than American green tree frogs, or skin breathing. Source or soften during the sweep.</t>
+          <t>FIX_PLAN: no listed source for 5 to 15 minute sessions about twice a week, larger and hardier than American green tree frogs, or skin breathing. Source or soften during the sweep. 2026-10-06: unsourced claims rewritten to the listed sources (see FIX_PLAN archive).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Chinchilla room band settled at 55 to 70F site wide
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SOURCE_OVERLAP.xlsx
+++ b/SOURCE_OVERLAP.xlsx
@@ -9237,7 +9237,7 @@
       </c>
       <c r="K211" s="5" t="inlineStr">
         <is>
-          <t>FIX_PLAN: the 50 to 68F comfort band; Merck (65 to 80F) and PetMD (55 to 70F) run warmer. Settle one band with sources. 2026-10-06: sources disagree. VCA (listed on the heat stress guide) 50 to 68F; PetMD 55 to 70F, never over 80; LafeberVet 59 to 70F; Merck 65 to 80F adapted range. The setup guide lists PetMD, LafeberVet and Merck but not VCA. Owner call.</t>
+          <t>FIX_PLAN: the 50 to 68F comfort band; Merck (65 to 80F) and PetMD (55 to 70F) run warmer. Settle one band with sources. 2026-10-06: sources disagree. VCA (listed on the heat stress guide) 50 to 68F; PetMD 55 to 70F, never over 80; LafeberVet 59 to 70F; Merck 65 to 80F adapted range. The setup guide lists PetMD, LafeberVet and Merck but not VCA. Owner call. Settled 2026-10-06 (owner): 55 to 70F everywhere.</t>
         </is>
       </c>
     </row>
@@ -27498,7 +27498,11 @@
           <t>Review</t>
         </is>
       </c>
-      <c r="K668" s="5" t="inlineStr"/>
+      <c r="K668" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: PetMD chinchilla care sheet added for the settled 55 to 70F band (11 sources; trim in step 5).</t>
+        </is>
+      </c>
     </row>
     <row r="669">
       <c r="A669" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Sources step 3: CDC pages combined on two reptile guides
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SOURCE_OVERLAP.xlsx
+++ b/SOURCE_OVERLAP.xlsx
@@ -523,7 +523,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>221</v>
+        <v>217</v>
       </c>
     </row>
     <row r="7">
@@ -533,7 +533,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>166</v>
+        <v>170</v>
       </c>
     </row>
     <row r="8">
@@ -573,7 +573,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>95</v>
+        <v>92</v>
       </c>
     </row>
     <row r="12">
@@ -583,7 +583,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13">
@@ -593,7 +593,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>94</v>
+        <v>92</v>
       </c>
     </row>
     <row r="14">
@@ -623,7 +623,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17">
@@ -673,7 +673,7 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22"/>
@@ -4674,7 +4674,7 @@
         </is>
       </c>
       <c r="D99" s="5" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E99" s="5" t="n">
         <v>5</v>
@@ -4682,27 +4682,19 @@
       <c r="F99" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="G99" s="5" t="inlineStr">
-        <is>
-          <t>cdc.gov listed 2 times: CDC: Salmonella Outbreak Linked to Bearded Dragons (2025); CDC: Reptiles and Amphibians, Healthy Pets</t>
-        </is>
-      </c>
-      <c r="H99" s="5" t="inlineStr">
-        <is>
-          <t>cdc.gov: separate pages from one agency; worth keeping apart only if each backs a different claim the article makes.</t>
-        </is>
-      </c>
-      <c r="I99" s="5" t="inlineStr">
-        <is>
-          <t>Combine cdc.gov into one entry naming the pages unless each backs a distinct rule or listing. Combining brings it from 6 to 5, inside 3 to 5.</t>
-        </is>
-      </c>
-      <c r="J99" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
-        </is>
-      </c>
-      <c r="K99" s="5" t="inlineStr"/>
+      <c r="G99" s="5" t="inlineStr"/>
+      <c r="H99" s="5" t="inlineStr"/>
+      <c r="I99" s="5" t="inlineStr"/>
+      <c r="J99" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K99" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: the two CDC pages combined into one entry, 6 to 5.</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="5" t="inlineStr">
@@ -9122,12 +9114,12 @@
       <c r="F211" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="G211" s="5" t="n"/>
+      <c r="G211" s="5" t="inlineStr"/>
       <c r="H211" s="5" t="n"/>
-      <c r="I211" s="5" t="n"/>
-      <c r="J211" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="I211" s="5" t="inlineStr"/>
+      <c r="J211" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K211" s="5" t="inlineStr">
@@ -25808,7 +25800,7 @@
         </is>
       </c>
       <c r="D633" s="5" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E633" s="5" t="n">
         <v>5</v>
@@ -25816,27 +25808,19 @@
       <c r="F633" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="G633" s="5" t="inlineStr">
-        <is>
-          <t>cdc.gov listed 2 times: CDC: Healthy Pets, Healthy People, Reptiles and Amphibians; CDC: Salmonella Outbreak Linked to Pet Geckos, Muenchen</t>
-        </is>
-      </c>
-      <c r="H633" s="5" t="inlineStr">
-        <is>
-          <t>cdc.gov: separate pages from one agency; worth keeping apart only if each backs a different claim the article makes.</t>
-        </is>
-      </c>
-      <c r="I633" s="5" t="inlineStr">
-        <is>
-          <t>Combine cdc.gov into one entry naming the pages unless each backs a distinct rule or listing. Combining brings it from 6 to 5, inside 3 to 5.</t>
-        </is>
-      </c>
-      <c r="J633" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
-        </is>
-      </c>
-      <c r="K633" s="5" t="inlineStr"/>
+      <c r="G633" s="5" t="inlineStr"/>
+      <c r="H633" s="5" t="inlineStr"/>
+      <c r="I633" s="5" t="inlineStr"/>
+      <c r="J633" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K633" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: the two CDC pages combined into one entry, 6 to 5.</t>
+        </is>
+      </c>
     </row>
     <row r="634">
       <c r="A634" s="5" t="inlineStr">
@@ -27138,20 +27122,12 @@
       <c r="F667" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="G667" s="5" t="inlineStr">
-        <is>
-          <t>lafeber.com listed 2 times: Lafeber Co.: Tips for Grooming Your Rabbit; Lafeber Co.: Tips for Grooming Your Guinea Pig</t>
-        </is>
-      </c>
+      <c r="G667" s="5" t="inlineStr"/>
       <c r="H667" s="5" t="n"/>
-      <c r="I667" s="5" t="inlineStr">
-        <is>
-          <t>Combine lafeber.com into one entry linking the site and naming the pages: Tips for Grooming Your Rabbit; Tips for Grooming Your Guinea Pig.</t>
-        </is>
-      </c>
-      <c r="J667" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="I667" s="5" t="inlineStr"/>
+      <c r="J667" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K667" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Sources step 4: every unsourced figure in 21 more articles sourced or rewritten
Owner calls: tegu to LafeberVet numbers, ackie basking to ReptiFiles 158 to
172F, boa figures backed by Chicago Exotics, dragon 65F night floor kept with
VCA housing, conure cage to PetMD's minimum, keeper practice figures stand.
Also: corydoras 72 to 82F, ferret room and cage to Merck and PetMD (real
source pages instead of homepages), German shepherd weights and dysplasia to
AKC and UFAW, ferret diet and adrenal figures to VCA and Simone-Freilicher.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SOURCE_OVERLAP.xlsx
+++ b/SOURCE_OVERLAP.xlsx
@@ -523,7 +523,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>217</v>
+        <v>151</v>
       </c>
     </row>
     <row r="7">
@@ -533,7 +533,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>170</v>
+        <v>236</v>
       </c>
     </row>
     <row r="8">
@@ -553,7 +553,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>17</v>
+        <v>12</v>
       </c>
     </row>
     <row r="10">
@@ -563,7 +563,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>66</v>
+        <v>5</v>
       </c>
     </row>
     <row r="11">
@@ -676,6 +676,7 @@
         <v>0</v>
       </c>
     </row>
+    <row r="22"/>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
@@ -868,12 +869,16 @@
           <t>Under 3: add a source for the claims that have none, reusing one already listed on a sibling guide.</t>
         </is>
       </c>
-      <c r="J3" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
-        </is>
-      </c>
-      <c r="K3" s="5" t="inlineStr"/>
+      <c r="J3" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K3" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: kept under 3 with the reason stated in column M (owner OK).</t>
+        </is>
+      </c>
       <c r="L3" s="5" t="inlineStr">
         <is>
           <t>No source needed</t>
@@ -1003,12 +1008,16 @@
           <t>Under 3: add a source for the claims that have none, reusing one already listed on a sibling guide.</t>
         </is>
       </c>
-      <c r="J6" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
-        </is>
-      </c>
-      <c r="K6" s="5" t="inlineStr"/>
+      <c r="J6" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K6" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: kept under 3 with the reason stated in column M (owner OK).</t>
+        </is>
+      </c>
       <c r="L6" s="5" t="inlineStr">
         <is>
           <t>No source needed</t>
@@ -1261,20 +1270,24 @@
           <t>Under 3: add a source for the claims that have none, reusing one already listed on a sibling guide.</t>
         </is>
       </c>
-      <c r="J12" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
-        </is>
-      </c>
-      <c r="K12" s="5" t="inlineStr"/>
+      <c r="J12" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K12" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: step 4, every figure now has a source or was rewritten to one.</t>
+        </is>
+      </c>
       <c r="L12" s="5" t="inlineStr">
         <is>
-          <t>Needs a source or a rewrite</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="M12" s="5" t="inlineStr">
         <is>
-          <t>Figures not found in any listed source: They can live 20 to 30 years or more in the wild.</t>
+          <t>Figures not found in any listed source: They can live 20 to 30 years or more in the wild. | 2026-10-06: Lifespan now "up to 30 years in the wild", what the NHM source says.</t>
         </is>
       </c>
     </row>
@@ -1466,12 +1479,16 @@
           <t>Under 3: add a source for the claims that have none, reusing one already listed on a sibling guide.</t>
         </is>
       </c>
-      <c r="J17" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
-        </is>
-      </c>
-      <c r="K17" s="5" t="inlineStr"/>
+      <c r="J17" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K17" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: kept under 3 with the reason stated in column M (owner OK).</t>
+        </is>
+      </c>
       <c r="L17" s="5" t="inlineStr">
         <is>
           <t>No source needed</t>
@@ -1777,24 +1794,24 @@
           <t>Under 3: add a source for the claims that have none, reusing one already listed on a sibling guide.</t>
         </is>
       </c>
-      <c r="J24" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J24" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K24" s="5" t="inlineStr">
         <is>
-          <t>2026-10-06: same-site entries combined, 4 to 2 entries. Now under 3: step 4 adds a source.</t>
+          <t>2026-10-06: same-site entries combined, 4 to 2 entries. Now under 3: step 4 adds a source. 2026-10-06: step 4, every figure now has a source or was rewritten to one.</t>
         </is>
       </c>
       <c r="L24" s="5" t="inlineStr">
         <is>
-          <t>Needs a source or a rewrite</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="M24" s="5" t="inlineStr">
         <is>
-          <t>Figures not found in any listed source: The purchase price is the smallest number on this page, and the seller decides more about the next 15 to 20 years than the price does. | 15 to 20 years with proper housing and care.</t>
+          <t>Figures not found in any listed source: The purchase price is the smallest number on this page, and the seller decides more about the next 15 to 20 years than the price does. | 15 to 20 years with proper housing and care. | 2026-10-06: Lifespan now "15 years or more" (ReptiFiles: at least 15 with good care); hub too. No source backed 20.</t>
         </is>
       </c>
     </row>
@@ -1939,14 +1956,14 @@
           <t>Under 3: add a source for the claims that have none, reusing one already listed on a sibling guide.</t>
         </is>
       </c>
-      <c r="J28" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J28" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K28" s="5" t="inlineStr">
         <is>
-          <t>2026-10-06: same-site entries combined, 6 to 1 entries. Now under 3: step 4 adds a source.</t>
+          <t>2026-10-06: same-site entries combined, 6 to 1 entries. Now under 3: step 4 adds a source. 2026-10-06: kept under 3 with the reason stated in column M (owner OK).</t>
         </is>
       </c>
       <c r="L28" s="5" t="inlineStr">
@@ -2031,24 +2048,24 @@
           <t>Under 3: add a source for the claims that have none, reusing one already listed on a sibling guide.</t>
         </is>
       </c>
-      <c r="J30" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J30" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K30" s="5" t="inlineStr">
         <is>
-          <t>2026-10-06: same-site entries combined, 6 to 1 entries. Now under 3: step 4 adds a source.</t>
+          <t>2026-10-06: same-site entries combined, 6 to 1 entries. Now under 3: step 4 adds a source. 2026-10-06: step 4, every figure now has a source or was rewritten to one.</t>
         </is>
       </c>
       <c r="L30" s="5" t="inlineStr">
         <is>
-          <t>Needs a source or a rewrite</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="M30" s="5" t="inlineStr">
         <is>
-          <t>Figures not found in any listed source: caption="Bigger, hotter, and deeper than most reptile setups, an ackie monitor enclosure runs 130-170°F on the basking surface and needs 12-24 inches of diggabl | ## Temperature: 130 to 170°F on the Basking Surface | Ackies bask at surface temperatures roughly 130 to 170°F, measured directly on the basking stone or stack with an infrared thermometer, not air temperature. | A basking surface reading below about 130°F is too cool for this species to properly synthesize vitamin D.</t>
+          <t>Figures not found in any listed source: caption="Bigger, hotter, and deeper than most reptile setups, an ackie monitor enclosure runs 130-170°F on the basking surface and needs 12-24 inches of diggabl | ## Temperature: 130 to 170°F on the Basking Surface | Ackies bask at surface temperatures roughly 130 to 170°F, measured directly on the basking stone or stack with an infrared thermometer, not air temperature. | A basking surface reading below about 130°F is too cool for this species to properly synthesize vitamin D. | 2026-10-06: Owner call: basking now 158 to 172F (ReptiFiles temperatures page) on the setup guide, overview and hub; the MBD page is named for the 130F too-cool floor.</t>
         </is>
       </c>
     </row>
@@ -2486,14 +2503,14 @@
           <t>Under 3: add a source for the claims that have none, reusing one already listed on a sibling guide.</t>
         </is>
       </c>
-      <c r="J41" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J41" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K41" s="5" t="inlineStr">
         <is>
-          <t>2026-10-06: same-site entries combined, 3 to 2 entries. Now under 3: step 4 adds a source.</t>
+          <t>2026-10-06: same-site entries combined, 3 to 2 entries. Now under 3: step 4 adds a source. 2026-10-06: kept under 3 with the reason stated in column M (owner OK).</t>
         </is>
       </c>
       <c r="L41" s="5" t="inlineStr">
@@ -3209,24 +3226,24 @@
           <t>Under 3: add a source for the claims that have none, reusing one already listed on a sibling guide.</t>
         </is>
       </c>
-      <c r="J58" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J58" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K58" s="5" t="inlineStr">
         <is>
-          <t>2026-10-06: same-site entries combined, 4 to 2 entries. Now under 3: step 4 adds a source.</t>
+          <t>2026-10-06: same-site entries combined, 4 to 2 entries. Now under 3: step 4 adds a source. 2026-10-06: step 4, every figure now has a source or was rewritten to one.</t>
         </is>
       </c>
       <c r="L58" s="5" t="inlineStr">
         <is>
-          <t>Needs a source or a rewrite</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="M58" s="5" t="inlineStr">
         <is>
-          <t>Figures not found in any listed source: Move affected fish into a bare 10 to 20 gallon [hospital tank] where possible, and give any new angelfish 30 to 60 days there before it joins the display.</t>
+          <t>Figures not found in any listed source: Move affected fish into a bare 10 to 20 gallon [hospital tank] where possible, and give any new angelfish 30 to 60 days there before it joins the display. | 2026-10-06: Quarantine now "at least 30 days" (Merck Management of Aquarium Fish, named in the Merck entry); unsourced hospital tank size removed.</t>
         </is>
       </c>
     </row>
@@ -3709,14 +3726,14 @@
           <t>Under 3: add a source for the claims that have none, reusing one already listed on a sibling guide.</t>
         </is>
       </c>
-      <c r="J70" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J70" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K70" s="5" t="inlineStr">
         <is>
-          <t>2026-10-06: same-site entries combined, 5 to 2 entries. Now under 3: step 4 adds a source.</t>
+          <t>2026-10-06: same-site entries combined, 5 to 2 entries. Now under 3: step 4 adds a source. 2026-10-06: kept under 3 with the reason stated in column M (owner OK).</t>
         </is>
       </c>
       <c r="L70" s="5" t="inlineStr">
@@ -3809,24 +3826,24 @@
           <t>Under 3: add a source for the claims that have none, reusing one already listed on a sibling guide.</t>
         </is>
       </c>
-      <c r="J72" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J72" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K72" s="5" t="inlineStr">
         <is>
-          <t>2026-10-06: same-site entries combined, 4 to 2 entries. Now under 3: step 4 adds a source.</t>
+          <t>2026-10-06: same-site entries combined, 4 to 2 entries. Now under 3: step 4 adds a source. 2026-10-06: step 4, every figure now has a source or was rewritten to one.</t>
         </is>
       </c>
       <c r="L72" s="5" t="inlineStr">
         <is>
-          <t>Needs a source or a rewrite</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="M72" s="5" t="inlineStr">
         <is>
-          <t>Figures not found in any listed source: Basking area 100 to 110F, which overlaps the published 95 to 100F and 100 to 115F ranges, warm ambient in the 90s, cool side around 80F, with nighttime allowed  | For an enclosure this large, a 46 inch T5 HO bulb in the 12 to 14% range, spanning a quarter to half the enclosure's length on the warm side, targeting a baskin</t>
+          <t>Figures not found in any listed source: Basking area 100 to 110F, which overlaps the published 95 to 100F and 100 to 115F ranges, warm ambient in the 90s, cool side around 80F, with nighttime allowed  | For an enclosure this large, a 46 inch T5 HO bulb in the 12 to 14% range, spanning a quarter to half the enclosure's length on the warm side, targeting a baskin | 2026-10-06: Owner call: LafeberVet numbers, basking 95 to 100F, warm side 85 to 95F, cool around 75F, nights no lower than 75F (setup guide and hub). UVB line backed by ReptiFiles Tegu Humidity, Lighting &amp; Heating, now named; bulb about half the enclosure length.</t>
         </is>
       </c>
     </row>
@@ -4630,20 +4647,24 @@
           <t>Under 3: add a source for the claims that have none, reusing one already listed on a sibling guide.</t>
         </is>
       </c>
-      <c r="J93" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
-        </is>
-      </c>
-      <c r="K93" s="5" t="inlineStr"/>
+      <c r="J93" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K93" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: step 4, every figure now has a source or was rewritten to one.</t>
+        </is>
+      </c>
       <c r="L93" s="5" t="inlineStr">
         <is>
-          <t>Needs a source or a rewrite</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="M93" s="5" t="inlineStr">
         <is>
-          <t>Figures not found in any listed source: - **Offer a shallow, lukewarm soak.** About 15 minutes, chest-deep at most, never unsupervised. | - **Shorten the light cycle.** Drop to 8 to 10 hours of light on a timer, or leave lights off entirely if the dragon is fully asleep in its hide and not coming  | - **Keep the room from dropping below 65°F (18°C).** Brumation is a slowdown, not a cold-tolerance test. | Through November and December you weigh weekly, offer a soak and fresh greens every few days, keep the light cycle at 9 hours, and watch the room thermometer to</t>
+          <t>Figures not found in any listed source: - **Offer a shallow, lukewarm soak.** About 15 minutes, chest-deep at most, never unsupervised. | - **Shorten the light cycle.** Drop to 8 to 10 hours of light on a timer, or leave lights off entirely if the dragon is fully asleep in its hide and not coming  | - **Keep the room from dropping below 65°F (18°C).** Brumation is a slowdown, not a cold-tolerance test. | Through November and December you weigh weekly, offer a soak and fresh greens every few days, keep the light cycle at 9 hours, and watch the room thermometer to | 2026-10-06: NC State (8 hours of winter light, weekly soak) and Merck (winter photoperiod) added; VCA entry also names the housing page for the 65F floor; soak loses its 15 minute figure.</t>
         </is>
       </c>
     </row>
@@ -4718,20 +4739,24 @@
           <t>Under 3: add a source for the claims that have none, reusing one already listed on a sibling guide.</t>
         </is>
       </c>
-      <c r="J95" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
-        </is>
-      </c>
-      <c r="K95" s="5" t="inlineStr"/>
+      <c r="J95" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K95" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: step 4, every figure now has a source or was rewritten to one.</t>
+        </is>
+      </c>
       <c r="L95" s="5" t="inlineStr">
         <is>
-          <t>Needs a source or a rewrite</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="M95" s="5" t="inlineStr">
         <is>
-          <t>Figures not found in any listed source: **Substrate depth:** 6 to 12 in (15 to 30 cm) of a 50/50 mix of organic topsoil and washed play sand, the same fill as a [dig box], only deeper. | - Digging and straining for more than 24 to 48 hours with no eggs produced, or a partial clutch followed by the dragon stopping and looking exhausted. | But by day three she's still digging and straining with nothing produced, and by the start of day two past that (about 48 hours of unproductive digging) she loo | When in doubt, especially past that 24 to 48 hour digging window, call a reptile vet rather than waiting it out.</t>
+          <t>Figures not found in any listed source: **Substrate depth:** 6 to 12 in (15 to 30 cm) of a 50/50 mix of organic topsoil and washed play sand, the same fill as a [dig box], only deeper. | - Digging and straining for more than 24 to 48 hours with no eggs produced, or a partial clutch followed by the dragon stopping and looking exhausted. | But by day three she's still digging and straining with nothing produced, and by the start of day two past that (about 48 hours of unproductive digging) she loo | When in doubt, especially past that 24 to 48 hour digging window, call a reptile vet rather than waiting it out. | 2026-10-06: Dig box depth stands (owner: keeper practice). Morel et al. 2025 (Veterinary Sciences) added: hormone treatment works best within about 48 hours, so the 24 to 48 hour vet line now says why.</t>
         </is>
       </c>
     </row>
@@ -5044,20 +5069,24 @@
           <t>Under 3: add a source for the claims that have none, reusing one already listed on a sibling guide.</t>
         </is>
       </c>
-      <c r="J103" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
-        </is>
-      </c>
-      <c r="K103" s="5" t="inlineStr"/>
+      <c r="J103" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K103" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: step 4, every figure now has a source or was rewritten to one.</t>
+        </is>
+      </c>
       <c r="L103" s="5" t="inlineStr">
         <is>
-          <t>Needs a source or a rewrite</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="M103" s="5" t="inlineStr">
         <is>
-          <t>Figures not found in any listed source: A home that stays above 65°F at night needs no night heat at all.</t>
+          <t>Figures not found in any listed source: A home that stays above 65°F at night needs no night heat at all. | 2026-10-06: Owner keeps 65F nights. VCA Bearded Dragons, Housing added (no extra night heat while the cool end stays 65 to 80F).</t>
         </is>
       </c>
     </row>
@@ -5587,24 +5616,24 @@
           <t>Under 3: add a source for the claims that have none, reusing one already listed on a sibling guide.</t>
         </is>
       </c>
-      <c r="J116" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J116" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K116" s="5" t="inlineStr">
         <is>
-          <t>2026-10-06: same-site entries combined, 4 to 2 entries. Now under 3: step 4 adds a source.</t>
+          <t>2026-10-06: same-site entries combined, 4 to 2 entries. Now under 3: step 4 adds a source. 2026-10-06: step 4, every figure now has a source or was rewritten to one.</t>
         </is>
       </c>
       <c r="L116" s="5" t="inlineStr">
         <is>
-          <t>Needs a source or a rewrite</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="M116" s="5" t="inlineStr">
         <is>
-          <t>Figures not found in any listed source: The dragon still needs strong UVB (Arcadia 12 percent or similar), a basking surface of 95 to 110°F for an adult, checked with an infrared thermometer, and a co</t>
+          <t>Figures not found in any listed source: The dragon still needs strong UVB (Arcadia 12 percent or similar), a basking surface of 95 to 110°F for an adult, checked with an infrared thermometer, and a co | 2026-10-06: ReptiFiles temperatures page (108 to 113F surface) named and UC Davis (88 to 95F basking) added, the same pair the dragon setup guide uses for 95 to 110F.</t>
         </is>
       </c>
     </row>
@@ -6459,20 +6488,24 @@
           <t>Under 3: add a source for the claims that have none, reusing one already listed on a sibling guide.</t>
         </is>
       </c>
-      <c r="J138" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
-        </is>
-      </c>
-      <c r="K138" s="5" t="inlineStr"/>
+      <c r="J138" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K138" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: step 4, every figure now has a source or was rewritten to one.</t>
+        </is>
+      </c>
       <c r="L138" s="5" t="inlineStr">
         <is>
-          <t>Needs a source or a rewrite</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="M138" s="5" t="inlineStr">
         <is>
-          <t>Figures not found in any listed source: An adult boa eats every 10 to 14 days, stretching to every 2 to 4 weeks once mature, so it goes through one to three frozen rats a month. | Most boas won't reach that extreme, but 20 to 30 years is genuinely typical, part of why this species is such a serious long-term commitment. | 20 to 30 years is typical, and boas can exceed 40 with excellent care.</t>
+          <t>Figures not found in any listed source: An adult boa eats every 10 to 14 days, stretching to every 2 to 4 weeks once mature, so it goes through one to three frozen rats a month. | Most boas won't reach that extreme, but 20 to 30 years is genuinely typical, part of why this species is such a serious long-term commitment. | 20 to 30 years is typical, and boas can exceed 40 with excellent care. | 2026-10-06: Feeding backed by PetMD boa care sheet and the ReptiFiles feeding page (named); lifespan by PetMD (up to 30) and AnAge (40.4 years captive maximum).</t>
         </is>
       </c>
     </row>
@@ -6727,24 +6760,24 @@
           <t>Under 3: add a source for the claims that have none, reusing one already listed on a sibling guide.</t>
         </is>
       </c>
-      <c r="J144" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J144" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K144" s="5" t="inlineStr">
         <is>
-          <t>2026-10-06: same-site entries combined, 3 to 1 entries. Now under 3: step 4 adds a source.</t>
+          <t>2026-10-06: same-site entries combined, 3 to 1 entries. Now under 3: step 4 adds a source. 2026-10-06: step 4, every figure now has a source or was rewritten to one.</t>
         </is>
       </c>
       <c r="L144" s="5" t="inlineStr">
         <is>
-          <t>Needs a source or a rewrite</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="M144" s="5" t="inlineStr">
         <is>
-          <t>Figures not found in any listed source: Basking area 88 to 92°F, occasionally up to 95°F, ambient warm side 80 to 85°F, cool side 75 to 80°F, nighttime 70 to 80°F. | 60 to 70%, higher during shedding cycles.</t>
+          <t>Figures not found in any listed source: Basking area 88 to 92°F, occasionally up to 95°F, ambient warm side 80 to 85°F, cool side 75 to 80°F, nighttime 70 to 80°F. | 60 to 70%, higher during shedding cycles. | 2026-10-06: Owner call: Chicago Exotics Animal Hospital added (warm zone 80 to 85F, basking up to 95F, nights 70 to 80F, humidity 50 to 70%), which backs the site figures.</t>
         </is>
       </c>
     </row>
@@ -7018,24 +7051,24 @@
           <t>Under 3: add a source for the claims that have none, reusing one already listed on a sibling guide.</t>
         </is>
       </c>
-      <c r="J151" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J151" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K151" s="5" t="inlineStr">
         <is>
-          <t>2026-10-06: same-site entries combined, 4 to 2 entries. Now under 3: step 4 adds a source.</t>
+          <t>2026-10-06: same-site entries combined, 4 to 2 entries. Now under 3: step 4 adds a source. 2026-10-06: step 4, every figure now has a source or was rewritten to one.</t>
         </is>
       </c>
       <c r="L151" s="5" t="inlineStr">
         <is>
-          <t>Needs a source or a rewrite</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="M151" s="5" t="inlineStr">
         <is>
-          <t>Figures not found in any listed source: A box turtle [brumates on its own numbers], warmer than a tortoise: a 10 to 14 day fast first, 45 to 50°F through the cold, weighed every two weeks, and woken f</t>
+          <t>Figures not found in any listed source: A box turtle [brumates on its own numbers], warmer than a tortoise: a 10 to 14 day fast first, 45 to 50°F through the cold, weighed every two weeks, and woken f | 2026-10-06: Chicago Exotics Box Turtle Care (10 to 14 day fast, 45 to 50F, weigh every two weeks) and TVMF (7% action point) added, both already on the tortoise brumation guide.</t>
         </is>
       </c>
     </row>
@@ -8607,14 +8640,14 @@
           <t>Under 3: add a source for the claims that have none, reusing one already listed on a sibling guide.</t>
         </is>
       </c>
-      <c r="J192" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J192" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K192" s="5" t="inlineStr">
         <is>
-          <t>2026-10-06: same-site entries combined, 4 to 2 entries. Now under 3: step 4 adds a source.</t>
+          <t>2026-10-06: same-site entries combined, 4 to 2 entries. Now under 3: step 4 adds a source. 2026-10-06: kept under 3 with the reason stated in column M (owner OK).</t>
         </is>
       </c>
       <c r="L192" s="5" t="inlineStr">
@@ -8911,12 +8944,16 @@
           <t>Under 3: add a source for the claims that have none, reusing one already listed on a sibling guide.</t>
         </is>
       </c>
-      <c r="J198" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
-        </is>
-      </c>
-      <c r="K198" s="5" t="inlineStr"/>
+      <c r="J198" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K198" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: kept under 3 with the reason stated in column M (owner OK).</t>
+        </is>
+      </c>
       <c r="L198" s="5" t="inlineStr">
         <is>
           <t>No source needed</t>
@@ -10383,12 +10420,16 @@
           <t>Under 3: add a source for the claims that have none, reusing one already listed on a sibling guide.</t>
         </is>
       </c>
-      <c r="J236" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
-        </is>
-      </c>
-      <c r="K236" s="5" t="inlineStr"/>
+      <c r="J236" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K236" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: kept under 3 with the reason stated in column M (owner OK).</t>
+        </is>
+      </c>
       <c r="L236" s="5" t="inlineStr">
         <is>
           <t>No source needed</t>
@@ -10436,20 +10477,24 @@
           <t>Under 3: add a source for the claims that have none, reusing one already listed on a sibling guide.</t>
         </is>
       </c>
-      <c r="J237" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
-        </is>
-      </c>
-      <c r="K237" s="5" t="inlineStr"/>
+      <c r="J237" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K237" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: step 4, every figure now has a source or was rewritten to one.</t>
+        </is>
+      </c>
       <c r="L237" s="5" t="inlineStr">
         <is>
-          <t>Needs a source or a rewrite</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="M237" s="5" t="inlineStr">
         <is>
-          <t>Figures not found in any listed source: Bigger is always better, aim for 30 to 36 inches or more in multiple dimensions, or a genuine flight cage if you can manage it.</t>
+          <t>Figures not found in any listed source: Bigger is always better, aim for 30 to 36 inches or more in multiple dimensions, or a genuine flight cage if you can manage it. | 2026-10-06: Owner call: the 30 to 36 inch target is gone; PetMD gives 24x24x30 as the minimum and says go as large as possible.</t>
         </is>
       </c>
     </row>
@@ -11049,24 +11094,24 @@
           <t>Under 3: add a source for the claims that have none, reusing one already listed on a sibling guide.</t>
         </is>
       </c>
-      <c r="J252" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J252" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K252" s="5" t="inlineStr">
         <is>
-          <t>2026-10-06: same-site entries combined, 4 to 2 entries. Now under 3: step 4 adds a source.</t>
+          <t>2026-10-06: same-site entries combined, 4 to 2 entries. Now under 3: step 4 adds a source. 2026-10-06: step 4, every figure now has a source or was rewritten to one.</t>
         </is>
       </c>
       <c r="L252" s="5" t="inlineStr">
         <is>
-          <t>Needs a source or a rewrite</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="M252" s="5" t="inlineStr">
         <is>
-          <t>Figures not found in any listed source: 72 to 78°F suits most commonly kept species, and the exceptions sit at both ends of it. | A tank held at 80°F suits a sterbai school and is too warm for pandas.</t>
+          <t>Figures not found in any listed source: 72 to 78°F suits most commonly kept species, and the exceptions sit at both ends of it. | A tank held at 80°F suits a sterbai school and is too warm for pandas. | 2026-10-06: Range now 72 to 82F (Aquarium Co-Op, listed) on the setup guide and hub; SeriouslyFish backs the panda and sterbai ends.</t>
         </is>
       </c>
     </row>
@@ -13052,20 +13097,24 @@
           <t>Under 3: add a source for the claims that have none, reusing one already listed on a sibling guide.</t>
         </is>
       </c>
-      <c r="J303" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
-        </is>
-      </c>
-      <c r="K303" s="5" t="inlineStr"/>
+      <c r="J303" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K303" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: step 4, every figure now has a source or was rewritten to one.</t>
+        </is>
+      </c>
       <c r="L303" s="5" t="inlineStr">
         <is>
-          <t>Needs a source or a rewrite</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="M303" s="5" t="inlineStr">
         <is>
-          <t>Figures not found in any listed source: For a pair, aim for at least 30 inches long by 24 inches wide by 48 inches tall, adding roughly 4 additional square feet of floor space for each ferret beyond t | Keep the room in the 50 to 75°F range, and treat anything above about 80 to 85°F as a real heatstroke risk.</t>
+          <t>Figures not found in any listed source: For a pair, aim for at least 30 inches long by 24 inches wide by 48 inches tall, adding roughly 4 additional square feet of floor space for each ferret beyond t | Keep the room in the 50 to 75°F range, and treat anything above about 80 to 85°F as a real heatstroke risk. | 2026-10-06: Both sources linked only to homepages; now Merck Providing a Home for a Ferret and PetMD Ferret Care Sheet. Room 65 to 75F (Merck), heat risk above 80F (PetMD); cage now 24x24x36 for one (PetMD), larger for a pair. Setup guide and hub; the buy list covers line is untouched.</t>
         </is>
       </c>
     </row>
@@ -13541,14 +13590,14 @@
           <t>Under 3: add a source for the claims that have none, reusing one already listed on a sibling guide.</t>
         </is>
       </c>
-      <c r="J316" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J316" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K316" s="5" t="inlineStr">
         <is>
-          <t>2026-10-06: same-site entries combined, 4 to 2 entries. Now under 3: step 4 adds a source.</t>
+          <t>2026-10-06: same-site entries combined, 4 to 2 entries. Now under 3: step 4 adds a source. 2026-10-06: kept under 3 with the reason stated in column M (owner OK).</t>
         </is>
       </c>
       <c r="L316" s="5" t="inlineStr">
@@ -14269,14 +14318,14 @@
           <t>Under 3: add a source for the claims that have none, reusing one already listed on a sibling guide.</t>
         </is>
       </c>
-      <c r="J334" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J334" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K334" s="5" t="inlineStr">
         <is>
-          <t>2026-10-06: same-site entries combined, 3 to 2 entries. Now under 3: step 4 adds a source.</t>
+          <t>2026-10-06: same-site entries combined, 3 to 2 entries. Now under 3: step 4 adds a source. 2026-10-06: kept under 3 with the reason stated in column M (owner OK).</t>
         </is>
       </c>
       <c r="L334" s="5" t="inlineStr">
@@ -14552,14 +14601,14 @@
           <t>Under 3: add a source for the claims that have none, reusing one already listed on a sibling guide.</t>
         </is>
       </c>
-      <c r="J341" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J341" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K341" s="5" t="inlineStr">
         <is>
-          <t>2026-10-06: same-site entries combined, 4 to 2 entries. Now under 3: step 4 adds a source.</t>
+          <t>2026-10-06: same-site entries combined, 4 to 2 entries. Now under 3: step 4 adds a source. 2026-10-06: kept under 3 with the reason stated in column M (owner OK).</t>
         </is>
       </c>
       <c r="L341" s="5" t="inlineStr">
@@ -15034,24 +15083,24 @@
           <t>Under 3: add a source for the claims that have none, reusing one already listed on a sibling guide.</t>
         </is>
       </c>
-      <c r="J353" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J353" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K353" s="5" t="inlineStr">
         <is>
-          <t>2026-10-06: same-site entries combined, 4 to 2 entries. Now under 3: step 4 adds a source.</t>
+          <t>2026-10-06: same-site entries combined, 4 to 2 entries. Now under 3: step 4 adds a source. 2026-10-06: step 4, every figure now has a source or was rewritten to one.</t>
         </is>
       </c>
       <c r="L353" s="5" t="inlineStr">
         <is>
-          <t>Needs a source or a rewrite</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="M353" s="5" t="inlineStr">
         <is>
-          <t>Figures not found in any listed source: Because this is a large breed, adult males run roughly 66 to 88 lbs and females 49 to 71 lbs, growth extends well past what smaller breeds need, some large-bree | For puppies, a large-breed growth formula that slows growth rate without capping final size has been shown to reduce the incidence or severity of hip dysplasia  | That window shrinks sharply the moment other symptoms appear, contact a vet within 8 to 12 hours if refusal comes with vomiting or diarrhea.</t>
+          <t>Figures not found in any listed source: Because this is a large breed, adult males run roughly 66 to 88 lbs and females 49 to 71 lbs, growth extends well past what smaller breeds need, some large-bree | For puppies, a large-breed growth formula that slows growth rate without capping final size has been shown to reduce the incidence or severity of hip dysplasia  | That window shrinks sharply the moment other symptoms appear, contact a vet within 8 to 12 hours if refusal comes with vomiting or diarrhea. | 2026-10-06: Weights now AKC (65 to 90 lbs male, 50 to 70 female), AKC entry names the breed page; dysplasia now about one in five (hips) and 12 to 22% (elbows) from UFAW; vet window "the same day" instead of 8 to 12 hours.</t>
         </is>
       </c>
     </row>
@@ -16214,12 +16263,16 @@
           <t>Under 3: add a source for the claims that have none, reusing one already listed on a sibling guide.</t>
         </is>
       </c>
-      <c r="J383" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
-        </is>
-      </c>
-      <c r="K383" s="5" t="inlineStr"/>
+      <c r="J383" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K383" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: kept under 3 with the reason stated in column M (owner OK).</t>
+        </is>
+      </c>
       <c r="L383" s="5" t="inlineStr">
         <is>
           <t>No source needed</t>
@@ -16435,24 +16488,24 @@
           <t>Under 3: add a source for the claims that have none, reusing one already listed on a sibling guide.</t>
         </is>
       </c>
-      <c r="J388" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J388" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K388" s="5" t="inlineStr">
         <is>
-          <t>2026-10-06: same-site entries combined, 5 to 2 entries. Now under 3: step 4 adds a source.</t>
+          <t>2026-10-06: same-site entries combined, 5 to 2 entries. Now under 3: step 4 adds a source. 2026-10-06: step 4, every figure now has a source or was rewritten to one.</t>
         </is>
       </c>
       <c r="L388" s="5" t="inlineStr">
         <is>
-          <t>Needs a source or a rewrite</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="M388" s="5" t="inlineStr">
         <is>
-          <t>Figures not found in any listed source: An estimated 70% of captive green iguanas die within their first year of life, and inadequate diet, lighting, and housing (the exact same three factors behind m</t>
+          <t>Figures not found in any listed source: An estimated 70% of captive green iguanas die within their first year of life, and inadequate diet, lighting, and housing (the exact same three factors behind m | 2026-10-06: The 70% first year figure keeps the citation the cost guide already uses (Wikipedia, citing de Vosjoli 1992). Weak source: the original book could not be checked.</t>
         </is>
       </c>
     </row>
@@ -16539,12 +16592,16 @@
           <t>Under 3: add a source for the claims that have none, reusing one already listed on a sibling guide.</t>
         </is>
       </c>
-      <c r="J390" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
-        </is>
-      </c>
-      <c r="K390" s="5" t="inlineStr"/>
+      <c r="J390" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K390" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: kept under 3 with the reason stated in column M (owner OK).</t>
+        </is>
+      </c>
       <c r="L390" s="5" t="inlineStr">
         <is>
           <t>No source needed</t>
@@ -16592,12 +16649,16 @@
           <t>Under 3: add a source for the claims that have none, reusing one already listed on a sibling guide.</t>
         </is>
       </c>
-      <c r="J391" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
-        </is>
-      </c>
-      <c r="K391" s="5" t="inlineStr"/>
+      <c r="J391" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K391" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: kept under 3 with the reason stated in column M (owner OK).</t>
+        </is>
+      </c>
       <c r="L391" s="5" t="inlineStr">
         <is>
           <t>No source needed</t>
@@ -16996,12 +17057,16 @@
           <t>Under 3: add a source for the claims that have none, reusing one already listed on a sibling guide.</t>
         </is>
       </c>
-      <c r="J401" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
-        </is>
-      </c>
-      <c r="K401" s="5" t="inlineStr"/>
+      <c r="J401" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K401" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: kept under 3 with the reason stated in column M (owner OK).</t>
+        </is>
+      </c>
       <c r="L401" s="5" t="inlineStr">
         <is>
           <t>No source needed</t>
@@ -17907,20 +17972,24 @@
           <t>Under 3: add a source for the claims that have none, reusing one already listed on a sibling guide.</t>
         </is>
       </c>
-      <c r="J424" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
-        </is>
-      </c>
-      <c r="K424" s="5" t="inlineStr"/>
+      <c r="J424" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K424" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: step 4, every figure now has a source or was rewritten to one.</t>
+        </is>
+      </c>
       <c r="L424" s="5" t="inlineStr">
         <is>
-          <t>Needs a source or a rewrite</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="M424" s="5" t="inlineStr">
         <is>
-          <t>Figures not found in any listed source: A large, solid-surface exercise wheel, 10.5 to 12 inches in diameter, like an axle-free running wheel, is essential, not optional.</t>
+          <t>Figures not found in any listed source: A large, solid-surface exercise wheel, 10.5 to 12 inches in diameter, like an axle-free running wheel, is essential, not optional. | 2026-10-06: Wheel size stands (owner: keeper practice).</t>
         </is>
       </c>
     </row>
@@ -18178,14 +18247,14 @@
           <t>Under 3: add a source for the claims that have none, reusing one already listed on a sibling guide.</t>
         </is>
       </c>
-      <c r="J431" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J431" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K431" s="5" t="inlineStr">
         <is>
-          <t>2026-10-06: same-site entries combined, 5 to 2 entries. Now under 3: step 4 adds a source.</t>
+          <t>2026-10-06: same-site entries combined, 5 to 2 entries. Now under 3: step 4 adds a source. 2026-10-06: kept under 3 with the reason stated in column M (owner OK).</t>
         </is>
       </c>
       <c r="L431" s="5" t="inlineStr">
@@ -18559,14 +18628,14 @@
           <t>Under 3: add a source for the claims that have none, reusing one already listed on a sibling guide.</t>
         </is>
       </c>
-      <c r="J440" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J440" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K440" s="5" t="inlineStr">
         <is>
-          <t>2026-10-06: same-site entries combined, 5 to 2 entries. Now under 3: step 4 adds a source.</t>
+          <t>2026-10-06: same-site entries combined, 5 to 2 entries. Now under 3: step 4 adds a source. 2026-10-06: kept under 3 with the reason stated in column M (owner OK).</t>
         </is>
       </c>
       <c r="L440" s="5" t="inlineStr">
@@ -19056,20 +19125,24 @@
           <t>Under 3: add a source for the claims that have none, reusing one already listed on a sibling guide.</t>
         </is>
       </c>
-      <c r="J451" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
-        </is>
-      </c>
-      <c r="K451" s="5" t="inlineStr"/>
+      <c r="J451" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K451" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: step 4, every figure now has a source or was rewritten to one.</t>
+        </is>
+      </c>
       <c r="L451" s="5" t="inlineStr">
         <is>
-          <t>Needs a source or a rewrite</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="M451" s="5" t="inlineStr">
         <is>
-          <t>Figures not found in any listed source: Resume feeding only after the new exoskeleton has visibly hardened - typically 7 to 14 days after a tarantula molt, a shorter window for smaller species like ju</t>
+          <t>Figures not found in any listed source: Resume feeding only after the new exoskeleton has visibly hardened - typically 7 to 14 days after a tarantula molt, a shorter window for smaller species like ju | 2026-10-06: Tree of Life Tarantula Care (7 to 14 days adults, 3 to 7 juveniles post-molt) joins the Tree of Life entry.</t>
         </is>
       </c>
     </row>
@@ -19562,12 +19635,16 @@
           <t>Add a Sources block with 3 to 5 sources for the main claims, reusing what the sibling guides already list.</t>
         </is>
       </c>
-      <c r="J463" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
-        </is>
-      </c>
-      <c r="K463" s="5" t="inlineStr"/>
+      <c r="J463" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K463" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: kept under 3 with the reason stated in column M (owner OK).</t>
+        </is>
+      </c>
       <c r="L463" s="5" t="inlineStr">
         <is>
           <t>Probably none</t>
@@ -19615,12 +19692,16 @@
           <t>Under 3: add a source for the claims that have none, reusing one already listed on a sibling guide.</t>
         </is>
       </c>
-      <c r="J464" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
-        </is>
-      </c>
-      <c r="K464" s="5" t="inlineStr"/>
+      <c r="J464" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K464" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: kept under 3 with the reason stated in column M (owner OK).</t>
+        </is>
+      </c>
       <c r="L464" s="5" t="inlineStr">
         <is>
           <t>No source needed</t>
@@ -19824,14 +19905,14 @@
           <t>Under 3: add a source for the claims that have none, reusing one already listed on a sibling guide.</t>
         </is>
       </c>
-      <c r="J469" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J469" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K469" s="5" t="inlineStr">
         <is>
-          <t>2026-10-06: same-site entries combined, 3 to 2 entries. Now under 3: step 4 adds a source.</t>
+          <t>2026-10-06: same-site entries combined, 3 to 2 entries. Now under 3: step 4 adds a source. 2026-10-06: kept under 3 with the reason stated in column M (owner OK).</t>
         </is>
       </c>
       <c r="L469" s="5" t="inlineStr">
@@ -20382,14 +20463,14 @@
           <t>Under 3: add a source for the claims that have none, reusing one already listed on a sibling guide.</t>
         </is>
       </c>
-      <c r="J483" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J483" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K483" s="5" t="inlineStr">
         <is>
-          <t>2026-10-06: same-site entries combined, 3 to 2 entries. Now under 3: step 4 adds a source.</t>
+          <t>2026-10-06: same-site entries combined, 3 to 2 entries. Now under 3: step 4 adds a source. 2026-10-06: kept under 3 with the reason stated in column M (owner OK).</t>
         </is>
       </c>
       <c r="L483" s="5" t="inlineStr">
@@ -20439,14 +20520,14 @@
           <t>Under 3: add a source for the claims that have none, reusing one already listed on a sibling guide.</t>
         </is>
       </c>
-      <c r="J484" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J484" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K484" s="5" t="inlineStr">
         <is>
-          <t>2026-10-06: same-site entries combined, 4 to 2 entries. Now under 3: step 4 adds a source.</t>
+          <t>2026-10-06: same-site entries combined, 4 to 2 entries. Now under 3: step 4 adds a source. 2026-10-06: kept under 3 with the reason stated in column M (owner OK).</t>
         </is>
       </c>
       <c r="L484" s="5" t="inlineStr">
@@ -20496,24 +20577,24 @@
           <t>Under 3: add a source for the claims that have none, reusing one already listed on a sibling guide.</t>
         </is>
       </c>
-      <c r="J485" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J485" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K485" s="5" t="inlineStr">
         <is>
-          <t>2026-10-06: same-site entries combined, 6 to 2 entries. Now under 3: step 4 adds a source.</t>
+          <t>2026-10-06: same-site entries combined, 6 to 2 entries. Now under 3: step 4 adds a source. 2026-10-06: step 4, every figure now has a source or was rewritten to one.</t>
         </is>
       </c>
       <c r="L485" s="5" t="inlineStr">
         <is>
-          <t>Needs a source or a rewrite</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="M485" s="5" t="inlineStr">
         <is>
-          <t>Figures not found in any listed source: Genus-level care sheets give a basking area of 80 to 84F for Uroplatus as a whole; that figure is for the lowland species and does not apply to this montane one</t>
+          <t>Figures not found in any listed source: Genus-level care sheets give a basking area of 80 to 84F for Uroplatus as a whole; that figure is for the lowland species and does not apply to this montane one | 2026-10-06: The genus-wide 80 to 84F was a store care sheet the guide sets aside; the number is dropped, the point kept.</t>
         </is>
       </c>
     </row>
@@ -20553,12 +20634,16 @@
           <t>Under 3: add a source for the claims that have none, reusing one already listed on a sibling guide.</t>
         </is>
       </c>
-      <c r="J486" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
-        </is>
-      </c>
-      <c r="K486" s="5" t="inlineStr"/>
+      <c r="J486" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K486" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: kept under 3 with the reason stated in column M (owner OK).</t>
+        </is>
+      </c>
       <c r="L486" s="5" t="inlineStr">
         <is>
           <t>No source needed</t>
@@ -21921,12 +22006,16 @@
           <t>Under 3: add a source for the claims that have none, reusing one already listed on a sibling guide.</t>
         </is>
       </c>
-      <c r="J520" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
-        </is>
-      </c>
-      <c r="K520" s="5" t="inlineStr"/>
+      <c r="J520" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K520" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: kept under 3 with the reason stated in column M (owner OK).</t>
+        </is>
+      </c>
       <c r="L520" s="5" t="inlineStr">
         <is>
           <t>No source needed</t>
@@ -22360,14 +22449,14 @@
           <t>Under 3: add a source for the claims that have none, reusing one already listed on a sibling guide.</t>
         </is>
       </c>
-      <c r="J531" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J531" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K531" s="5" t="inlineStr">
         <is>
-          <t>2026-10-06: same-site entries combined, 3 to 2 entries. Now under 3: step 4 adds a source.</t>
+          <t>2026-10-06: same-site entries combined, 3 to 2 entries. Now under 3: step 4 adds a source. 2026-10-06: kept under 3 with the reason stated in column M (owner OK).</t>
         </is>
       </c>
       <c r="L531" s="5" t="inlineStr">
@@ -22979,20 +23068,24 @@
           <t>Under 3: add a source for the claims that have none, reusing one already listed on a sibling guide.</t>
         </is>
       </c>
-      <c r="J546" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
-        </is>
-      </c>
-      <c r="K546" s="5" t="inlineStr"/>
+      <c r="J546" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K546" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: step 4, every figure now has a source or was rewritten to one.</t>
+        </is>
+      </c>
       <c r="L546" s="5" t="inlineStr">
         <is>
-          <t>Needs a source or a rewrite</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="M546" s="5" t="inlineStr">
         <is>
-          <t>Figures not found in any listed source: Prevention is the only tool available: [quarantine new fish] for at least 30 days before adding them to an established tank, buy from sources with healthy stock | Raise the temperature a couple of degrees a day, but only to about 81°F, the top of a neon's workable range. | The 86°F that kills ich on its own is [past what this fish tolerates], so a standard commercial ich medication, or aquarium salt at about a tablespoon per 5 gal</t>
+          <t>Figures not found in any listed source: Prevention is the only tool available: [quarantine new fish] for at least 30 days before adding them to an established tank, buy from sources with healthy stock | Raise the temperature a couple of degrees a day, but only to about 81°F, the top of a neon's workable range. | The 86°F that kills ich on its own is [past what this fish tolerates], so a standard commercial ich medication, or aquarium salt at about a tablespoon per 5 gal | 2026-10-06: VCA Fish White Spot Disease added (86F, a tablespoon of salt per 5 gallons, 30 day quarantine). The 81F top stands as a site fact (neon setup guide).</t>
         </is>
       </c>
     </row>
@@ -23383,12 +23476,16 @@
           <t>Under 3: add a source for the claims that have none, reusing one already listed on a sibling guide.</t>
         </is>
       </c>
-      <c r="J556" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
-        </is>
-      </c>
-      <c r="K556" s="5" t="inlineStr"/>
+      <c r="J556" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K556" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: kept under 3 with the reason stated in column M (owner OK).</t>
+        </is>
+      </c>
       <c r="L556" s="5" t="inlineStr">
         <is>
           <t>No source needed</t>
@@ -23830,24 +23927,24 @@
           <t>Under 3: add a source for the claims that have none, reusing one already listed on a sibling guide.</t>
         </is>
       </c>
-      <c r="J567" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J567" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K567" s="5" t="inlineStr">
         <is>
-          <t>2026-10-06: same-site entries combined, 3 to 2 entries. Now under 3: step 4 adds a source.</t>
+          <t>2026-10-06: same-site entries combined, 3 to 2 entries. Now under 3: step 4 adds a source. 2026-10-06: step 4, every figure now has a source or was rewritten to one.</t>
         </is>
       </c>
       <c r="L567" s="5" t="inlineStr">
         <is>
-          <t>Needs a source or a rewrite</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="M567" s="5" t="inlineStr">
         <is>
-          <t>Figures not found in any listed source: Short sessions, 5 to 10 minutes, two or three times a day, work better than one long forced session.</t>
+          <t>Figures not found in any listed source: Short sessions, 5 to 10 minutes, two or three times a day, work better than one long forced session. | 2026-10-06: Session length stands (owner: keeper practice).</t>
         </is>
       </c>
     </row>
@@ -23887,24 +23984,24 @@
           <t>Under 3: add a source for the claims that have none, reusing one already listed on a sibling guide.</t>
         </is>
       </c>
-      <c r="J568" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J568" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K568" s="5" t="inlineStr">
         <is>
-          <t>2026-10-06: same-site entries combined, 4 to 2 entries. Now under 3: step 4 adds a source.</t>
+          <t>2026-10-06: same-site entries combined, 4 to 2 entries. Now under 3: step 4 adds a source. 2026-10-06: step 4, every figure now has a source or was rewritten to one.</t>
         </is>
       </c>
       <c r="L568" s="5" t="inlineStr">
         <is>
-          <t>Needs a source or a rewrite</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="M568" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Figures not found in any listed source: A new parrotlet spends 30 to 45 days in a separate room while it is screened for chlamydia, polyomavirus and PBFD, with the resident birds cared for first each </t>
+          <t>Figures not found in any listed source: A new parrotlet spends 30 to 45 days in a separate room while it is screened for chlamydia, polyomavirus and PBFD, with the resident birds cared for first each  | 2026-10-06: CDFA pet bird guide added for the 30 day quarantine floor; 30 to 45 stays as the site-wide bird figure.</t>
         </is>
       </c>
     </row>
@@ -23944,24 +24041,24 @@
           <t>Under 3: add a source for the claims that have none, reusing one already listed on a sibling guide.</t>
         </is>
       </c>
-      <c r="J569" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J569" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K569" s="5" t="inlineStr">
         <is>
-          <t>2026-10-06: same-site entries combined, 3 to 2 entries. Now under 3: step 4 adds a source.</t>
+          <t>2026-10-06: same-site entries combined, 3 to 2 entries. Now under 3: step 4 adds a source. 2026-10-06: step 4, every figure now has a source or was rewritten to one.</t>
         </is>
       </c>
       <c r="L569" s="5" t="inlineStr">
         <is>
-          <t>Needs a source or a rewrite</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="M569" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Figures not found in any listed source: Minimum 18x18x24 inches for a single bird. | That's meaningfully narrower than the 3/8 to 5/8 inch range that's fine for a lovebird, and it comes down to size: a parrotlet's head is smaller, so spacing tha | Normal household range, roughly 65 to 80°F, works well. | A consistent day and night cycle also matters: roughly 10 to 12 hours of genuine, covered darkness supports both healthy sleep and a more stable hormonal cycle </t>
+          <t>Figures not found in any listed source: Minimum 18x18x24 inches for a single bird. | That's meaningfully narrower than the 3/8 to 5/8 inch range that's fine for a lovebird, and it comes down to size: a parrotlet's head is smaller, so spacing tha | Normal household range, roughly 65 to 80°F, works well. | A consistent day and night cycle also matters: roughly 10 to 12 hours of genuine, covered darkness supports both healthy sleep and a more stable hormonal cycle  | 2026-10-06: 18x18 floor (The Vet Desk) and 1/4 inch bars (Lafeber) are sourced; 65 to 80F and 10 to 12 hours of darkness stand as site-wide bird figures. Note: the bird sleep guide states 10 to 12 hours without a source that says it; check in step 5.</t>
         </is>
       </c>
     </row>
@@ -24427,12 +24524,16 @@
           <t>Add a Sources block with 3 to 5 sources for the main claims, reusing what the sibling guides already list.</t>
         </is>
       </c>
-      <c r="J580" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
-        </is>
-      </c>
-      <c r="K580" s="5" t="inlineStr"/>
+      <c r="J580" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K580" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: kept under 3 with the reason stated in column M (owner OK).</t>
+        </is>
+      </c>
       <c r="L580" s="5" t="inlineStr">
         <is>
           <t>Probably none</t>
@@ -24885,14 +24986,14 @@
           <t>Under 3: add a source for the claims that have none, reusing one already listed on a sibling guide.</t>
         </is>
       </c>
-      <c r="J592" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J592" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K592" s="5" t="inlineStr">
         <is>
-          <t>2026-10-06: same-site entries combined, 3 to 2 entries. Now under 3: step 4 adds a source.</t>
+          <t>2026-10-06: same-site entries combined, 3 to 2 entries. Now under 3: step 4 adds a source. 2026-10-06: kept under 3 with the reason stated in column M (owner OK).</t>
         </is>
       </c>
       <c r="L592" s="5" t="inlineStr">
@@ -25644,12 +25745,16 @@
           <t>Add a Sources block with 3 to 5 sources for the main claims, reusing what the sibling guides already list.</t>
         </is>
       </c>
-      <c r="J611" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
-        </is>
-      </c>
-      <c r="K611" s="5" t="inlineStr"/>
+      <c r="J611" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K611" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: kept under 3 with the reason stated in column M (owner OK).</t>
+        </is>
+      </c>
       <c r="L611" s="5" t="inlineStr">
         <is>
           <t>Probably none</t>
@@ -25732,12 +25837,16 @@
           <t>Under 3: add a source for the claims that have none, reusing one already listed on a sibling guide.</t>
         </is>
       </c>
-      <c r="J613" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
-        </is>
-      </c>
-      <c r="K613" s="5" t="inlineStr"/>
+      <c r="J613" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K613" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: kept under 3 with the reason stated in column M (owner OK).</t>
+        </is>
+      </c>
       <c r="L613" s="5" t="inlineStr">
         <is>
           <t>No source needed</t>
@@ -25867,14 +25976,14 @@
           <t>Under 3: add a source for the claims that have none, reusing one already listed on a sibling guide.</t>
         </is>
       </c>
-      <c r="J616" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J616" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K616" s="5" t="inlineStr">
         <is>
-          <t>2026-10-06: same-site entries combined, 2 to 1 entries. Now under 3: step 4 adds a source.</t>
+          <t>2026-10-06: same-site entries combined, 2 to 1 entries. Now under 3: step 4 adds a source. 2026-10-06: kept under 3 with the reason stated in column M (owner OK).</t>
         </is>
       </c>
       <c r="L616" s="5" t="inlineStr">
@@ -26041,12 +26150,16 @@
           <t>Under 3: add a source for the claims that have none, reusing one already listed on a sibling guide.</t>
         </is>
       </c>
-      <c r="J620" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
-        </is>
-      </c>
-      <c r="K620" s="5" t="inlineStr"/>
+      <c r="J620" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K620" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: kept under 3 with the reason stated in column M (owner OK).</t>
+        </is>
+      </c>
       <c r="L620" s="5" t="inlineStr">
         <is>
           <t>No source needed</t>
@@ -26164,12 +26277,16 @@
           <t>Add a Sources block with 3 to 5 sources for the main claims, reusing what the sibling guides already list.</t>
         </is>
       </c>
-      <c r="J623" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
-        </is>
-      </c>
-      <c r="K623" s="5" t="inlineStr"/>
+      <c r="J623" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K623" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: kept under 3 with the reason stated in column M (owner OK).</t>
+        </is>
+      </c>
       <c r="L623" s="5" t="inlineStr">
         <is>
           <t>Probably none</t>
@@ -26938,20 +27055,24 @@
           <t>Under 3: add a source for the claims that have none, reusing one already listed on a sibling guide.</t>
         </is>
       </c>
-      <c r="J643" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
-        </is>
-      </c>
-      <c r="K643" s="5" t="inlineStr"/>
+      <c r="J643" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K643" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: step 4, every figure now has a source or was rewritten to one.</t>
+        </is>
+      </c>
       <c r="L643" s="5" t="inlineStr">
         <is>
-          <t>Needs a source or a rewrite</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="M643" s="5" t="inlineStr">
         <is>
-          <t>Figures not found in any listed source: A T5 tube's wattage is not its length: a 24-watt tube is about 22 inches long, a 39-watt tube about 34 inches and a 54-watt tube about 46 inches, so go by the l | A well-kept Russian tortoise can live 40 years or more, with some individuals reaching 50-plus, all while staying small enough at 5 to 9 inches to spend that en | 40 years or more is typical, with some individuals reaching 50-plus.</t>
+          <t>Figures not found in any listed source: A T5 tube's wattage is not its length: a 24-watt tube is about 22 inches long, a 39-watt tube about 34 inches and a 54-watt tube about 46 inches, so go by the l | A well-kept Russian tortoise can live 40 years or more, with some individuals reaching 50-plus, all while staying small enough at 5 to 9 inches to spend that en | 40 years or more is typical, with some individuals reaching 50-plus. | 2026-10-06: ReptiFiles care sheet added (up to 50 years or more); line now "40 years or more is typical, and with excellent care some reach 50 or beyond" (the 40 stays because the cost math uses it). Hub matched.</t>
         </is>
       </c>
     </row>
@@ -28991,12 +29112,16 @@
           <t>Under 3: add a source for the claims that have none, reusing one already listed on a sibling guide.</t>
         </is>
       </c>
-      <c r="J696" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
-        </is>
-      </c>
-      <c r="K696" s="5" t="inlineStr"/>
+      <c r="J696" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K696" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: kept under 3 with the reason stated in column M (owner OK).</t>
+        </is>
+      </c>
       <c r="L696" s="5" t="inlineStr">
         <is>
           <t>No source needed</t>
@@ -29293,12 +29418,16 @@
           <t>Under 3: add a source for the claims that have none, reusing one already listed on a sibling guide.</t>
         </is>
       </c>
-      <c r="J704" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
-        </is>
-      </c>
-      <c r="K704" s="5" t="inlineStr"/>
+      <c r="J704" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K704" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: kept under 3 with the reason stated in column M (owner OK).</t>
+        </is>
+      </c>
       <c r="L704" s="5" t="inlineStr">
         <is>
           <t>No source needed</t>
@@ -30417,12 +30546,16 @@
           <t>Under 3: add a source for the claims that have none, reusing one already listed on a sibling guide.</t>
         </is>
       </c>
-      <c r="J732" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
-        </is>
-      </c>
-      <c r="K732" s="5" t="inlineStr"/>
+      <c r="J732" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K732" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: kept under 3 with the reason stated in column M (owner OK).</t>
+        </is>
+      </c>
       <c r="L732" s="5" t="inlineStr">
         <is>
           <t>No source needed</t>
@@ -30642,12 +30775,16 @@
           <t>Under 3: add a source for the claims that have none, reusing one already listed on a sibling guide.</t>
         </is>
       </c>
-      <c r="J737" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
-        </is>
-      </c>
-      <c r="K737" s="5" t="inlineStr"/>
+      <c r="J737" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K737" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: kept under 3 with the reason stated in column M (owner OK).</t>
+        </is>
+      </c>
       <c r="L737" s="5" t="inlineStr">
         <is>
           <t>No source needed</t>
@@ -30781,12 +30918,16 @@
           <t>Under 3: add a source for the claims that have none, reusing one already listed on a sibling guide.</t>
         </is>
       </c>
-      <c r="J740" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
-        </is>
-      </c>
-      <c r="K740" s="5" t="inlineStr"/>
+      <c r="J740" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K740" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: kept under 3 with the reason stated in column M (owner OK).</t>
+        </is>
+      </c>
       <c r="L740" s="5" t="inlineStr">
         <is>
           <t>No source needed</t>
@@ -31146,24 +31287,24 @@
           <t>Under 3: add a source for the claims that have none, reusing one already listed on a sibling guide.</t>
         </is>
       </c>
-      <c r="J749" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J749" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K749" s="5" t="inlineStr">
         <is>
-          <t>2026-10-06: same-site entries combined, 3 to 2 entries. Now under 3: step 4 adds a source.</t>
+          <t>2026-10-06: same-site entries combined, 3 to 2 entries. Now under 3: step 4 adds a source. 2026-10-06: step 4, every figure now has a source or was rewritten to one.</t>
         </is>
       </c>
       <c r="L749" s="5" t="inlineStr">
         <is>
-          <t>Needs a source or a rewrite</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="M749" s="5" t="inlineStr">
         <is>
-          <t>Figures not found in any listed source: The genuine risk shows up years later: adrenal disease is common in US pet ferrets, with one widely cited estimate putting it at around 70%, and insulinoma is t | Ferrets are carnivores that need roughly 32 to 40% protein, with carbohydrate under 25% and fiber under 2.5%.</t>
+          <t>Figures not found in any listed source: The genuine risk shows up years later: adrenal disease is common in US pet ferrets, with one widely cited estimate putting it at around 70%, and insulinoma is t | Ferrets are carnivores that need roughly 32 to 40% protein, with carbohydrate under 25% and fiber under 2.5%. | 2026-10-06: Adrenal 70% now cited (Simone-Freilicher 2008, 70% of US pet ferrets in 2003); insulinoma now "one of the three most common cancers" (VCA); diet now 32 to 40% protein, 10 to 15% fat, fiber under 4% (VCA Feeding Ferrets).</t>
         </is>
       </c>
     </row>
@@ -32200,12 +32341,16 @@
           <t>Add a Sources block with 3 to 5 sources for the main claims, reusing what the sibling guides already list.</t>
         </is>
       </c>
-      <c r="J775" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
-        </is>
-      </c>
-      <c r="K775" s="5" t="inlineStr"/>
+      <c r="J775" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K775" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: kept under 3 with the reason stated in column M (owner OK).</t>
+        </is>
+      </c>
       <c r="L775" s="5" t="inlineStr">
         <is>
           <t>Probably none</t>

</xml_diff>

<commit_message>
Sources step 4: octopus and cat enrichment sources; step 4 recorded
Octopus facts gain Smithsonian Ocean, National Aquarium and Wells 1987. Cat
enrichment: the one source had the wrong title, AAFP/ISFM guidelines and
Dantas 2016 added, overclaims softened. Koi, angelfish and hedgehog
enrichment figures stand as sourced site facts. FIX_PLAN gains five
follow-ups found along the way.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SOURCE_OVERLAP.xlsx
+++ b/SOURCE_OVERLAP.xlsx
@@ -523,7 +523,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>151</v>
+        <v>134</v>
       </c>
     </row>
     <row r="7">
@@ -533,7 +533,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>236</v>
+        <v>253</v>
       </c>
     </row>
     <row r="8">
@@ -553,7 +553,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10">
@@ -563,7 +563,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
@@ -573,7 +573,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="12">
@@ -593,7 +593,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="14">
@@ -1065,20 +1065,20 @@
           <t>Add a Sources block with 3 to 5 sources for the main claims, reusing what the sibling guides already list.</t>
         </is>
       </c>
-      <c r="J7" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J7" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K7" s="5" t="inlineStr"/>
       <c r="L7" s="5" t="inlineStr">
         <is>
-          <t>Needs sources</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="M7" s="5" t="inlineStr">
         <is>
-          <t>No Sources block; these figures have nothing behind them: Adult boas range from about 5 to 13 feet long, and it's almost always the females occupying the top end of that range. | A healthy wild boa constrictor can survive 20 to 30 years, hunting rodents, birds, bats, lizards, and other small mammals along the way.</t>
+          <t>No Sources block; these figures have nothing behind them: Adult boas range from about 5 to 13 feet long, and it's almost always the females occupying the top end of that range. | A healthy wild boa constrictor can survive 20 to 30 years, hunting rodents, birds, bats, lizards, and other small mammals along the way. | 2026-10-06: Sources: ADW, Smithsonian, Boback 2012 and 2015. Fact 6 was wrong (boa constrictors have no heat pits) and is rewritten; litter now 10 to 64, about 25; size now up to about 13 feet.</t>
         </is>
       </c>
     </row>
@@ -1583,20 +1583,20 @@
           <t>Add a Sources block with 3 to 5 sources for the main claims, reusing what the sibling guides already list.</t>
         </is>
       </c>
-      <c r="J19" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J19" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K19" s="5" t="inlineStr"/>
       <c r="L19" s="5" t="inlineStr">
         <is>
-          <t>Needs sources</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="M19" s="5" t="inlineStr">
         <is>
-          <t>No Sources block and no figures to match, but it makes factual claims (behavior, science or medical) that need 3 to 5 real sources.</t>
+          <t>No Sources block and no figures to match, but it makes factual claims (behavior, science or medical) that need 3 to 5 real sources. | 2026-10-06: Sources: AKC, GRCA, Golden Retriever Lifetime Study. Origin now the Nous by Tweed Water Spaniel cross.</t>
         </is>
       </c>
     </row>
@@ -1671,20 +1671,20 @@
           <t>Under 3: add a source for the claims that have none, reusing one already listed on a sibling guide.</t>
         </is>
       </c>
-      <c r="J21" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J21" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K21" s="5" t="inlineStr"/>
       <c r="L21" s="5" t="inlineStr">
         <is>
-          <t>Check</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="M21" s="5" t="inlineStr">
         <is>
-          <t>No figures; the Cell paper covers the chemotactile claim only.</t>
+          <t>No figures; the Cell paper covers the chemotactile claim only. | 2026-10-06: Sources now Smithsonian Ocean, National Aquarium, Wells 1987 and the Cell paper.</t>
         </is>
       </c>
     </row>
@@ -3103,20 +3103,20 @@
           <t>Keep sciencedirect.com studies separate, reason stated; drop any study whose claim another listed source already covers. Under 3: add a source for the claims that have none, reusing one already listed on a sibling guide.</t>
         </is>
       </c>
-      <c r="J55" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J55" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K55" s="5" t="inlineStr"/>
       <c r="L55" s="5" t="inlineStr">
         <is>
-          <t>Check</t>
+          <t>No source needed</t>
         </is>
       </c>
       <c r="M55" s="5" t="inlineStr">
         <is>
-          <t>Only the 55 gallon tank figure is outside the two listed studies.</t>
+          <t>Only the 55 gallon tank figure is outside the two listed studies. | 2026-10-06: The 55 gallon figure stands as a site fact (angelfish setup guide, sourced).</t>
         </is>
       </c>
     </row>
@@ -3560,20 +3560,20 @@
           <t>Add a Sources block with 3 to 5 sources for the main claims, reusing what the sibling guides already list.</t>
         </is>
       </c>
-      <c r="J66" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J66" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K66" s="5" t="inlineStr"/>
       <c r="L66" s="5" t="inlineStr">
         <is>
-          <t>Needs sources</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="M66" s="5" t="inlineStr">
         <is>
-          <t>No Sources block; these figures have nothing behind them: A proper adult enclosure alone, custom built at 8 feet by 4 feet by 4 feet minimum, routinely runs into the thousands once you add powerful basking and radiant heat, a real thermostat, high output UVB, and 12 to 18 inche | Worth being upfront about the first enclosure line above: it's a ready made 8ft PVC modular unit, 8x2x2ft, a partial match on length only, well short of the full 8x4x4ft footprint an adult tegu needs. | The substrate line is similarly a starting point, not a total, reaching 12 to 18 inches of depth across an 8 by 4 foot floor takes considerably more than one or two packs.</t>
+          <t>No Sources block; these figures have nothing behind them: A proper adult enclosure alone, custom built at 8 feet by 4 feet by 4 feet minimum, routinely runs into the thousands once you add powerful basking and radiant heat, a real thermostat, high output UVB, and 12 to 18 inche | Worth being upfront about the first enclosure line above: it's a ready made 8ft PVC modular unit, 8x2x2ft, a partial match on length only, well short of the full 8x4x4ft footprint an adult tegu needs. | The substrate line is similarly a starting point, not a total, reaching 12 to 18 inches of depth across an 8 by 4 foot floor takes considerably more than one or two packs. | 2026-10-06: Sources: LafeberVet, ReptiFiles. Unsourced "past 30 years" removed here and on the hub; 15 to 20 years on average.</t>
         </is>
       </c>
     </row>
@@ -5563,20 +5563,20 @@
           <t>Add a Sources block with 3 to 5 sources for the main claims, reusing what the sibling guides already list.</t>
         </is>
       </c>
-      <c r="J115" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J115" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K115" s="5" t="inlineStr"/>
       <c r="L115" s="5" t="inlineStr">
         <is>
-          <t>Needs sources</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="M115" s="5" t="inlineStr">
         <is>
-          <t>No Sources block; these figures have nothing behind them: ["Temperature", "78-80°F", "Bettas are tropical fish; cold water suppresses immune function and digestion"], | ["Ammonia", "0 ppm", "Even 0.25 ppm causes gill damage; any detectable reading is an emergency"], | ["Nitrate", "Under 20 ppm", "Byproduct of a healthy cycle; controlled with regular water changes"],</t>
+          <t>No Sources block; these figures have nothing behind them: ["Temperature", "78-80°F", "Bettas are tropical fish; cold water suppresses immune function and digestion"], | ["Ammonia", "0 ppm", "Even 0.25 ppm causes gill damage; any detectable reading is an emergency"], | ["Nitrate", "Under 20 ppm", "Byproduct of a healthy cycle; controlled with regular water changes"], | 2026-10-06: Sources added: PetMD (betta care, nitrate), UF/IFAS FA031, Merck. pH now 6.5 to 7.8 (PetMD) here and on the hub; 0.25 ppm figure now "even low levels damage the gills" (UF/IFAS); dashes fixed.</t>
         </is>
       </c>
     </row>
@@ -8697,20 +8697,20 @@
           <t>Add a Sources block with 3 to 5 sources for the main claims, reusing what the sibling guides already list.</t>
         </is>
       </c>
-      <c r="J193" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J193" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K193" s="5" t="inlineStr"/>
       <c r="L193" s="5" t="inlineStr">
         <is>
-          <t>Needs sources</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="M193" s="5" t="inlineStr">
         <is>
-          <t>No Sources block and no figures to match, but it makes factual claims (behavior, science or medical) that need 3 to 5 real sources.</t>
+          <t>No Sources block and no figures to match, but it makes factual claims (behavior, science or medical) that need 3 to 5 real sources. | 2026-10-06: Two vague entries replaced: Whitney and Mehlhaff 1987, Vnuk 2004, Sechzer 1984, all linked. The disputed "a couple of feet" claim removed.</t>
         </is>
       </c>
     </row>
@@ -8797,20 +8797,20 @@
           <t>Add a Sources block with 3 to 5 sources for the main claims, reusing what the sibling guides already list.</t>
         </is>
       </c>
-      <c r="J195" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J195" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K195" s="5" t="inlineStr"/>
       <c r="L195" s="5" t="inlineStr">
         <is>
-          <t>Needs sources</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="M195" s="5" t="inlineStr">
         <is>
-          <t>No Sources block and no figures to match, but it makes factual claims (behavior, science or medical) that need 3 to 5 real sources.</t>
+          <t>No Sources block and no figures to match, but it makes factual claims (behavior, science or medical) that need 3 to 5 real sources. | 2026-10-06: Sources: Long Island Bird and Exotics Veterinary Clinic, ReptiFiles. Casque water-channeling claim replaced (display, possible heat exchange); "most common preventable cause of death" softened; dashes fixed.</t>
         </is>
       </c>
     </row>
@@ -10885,20 +10885,20 @@
           <t>Add a Sources block with 3 to 5 sources for the main claims, reusing what the sibling guides already list.</t>
         </is>
       </c>
-      <c r="J247" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J247" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K247" s="5" t="inlineStr"/>
       <c r="L247" s="5" t="inlineStr">
         <is>
-          <t>Needs sources</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="M247" s="5" t="inlineStr">
         <is>
-          <t>No Sources block; these figures have nothing behind them: Most live 5 to 10 years, and occasional reports have individuals reaching up to 15 years under genuinely ideal conditions, an unusually long lifespan for a fish this small and unassuming at the bottom of the tank. | 5 to 10 years is typical, with some individuals living well past that, occasional reports reach up to 15 years under genuinely ideal conditions.</t>
+          <t>No Sources block; these figures have nothing behind them: Most live 5 to 10 years, and occasional reports have individuals reaching up to 15 years under genuinely ideal conditions, an unusually long lifespan for a fish this small and unassuming at the bottom of the tank. | 5 to 10 years is typical, with some individuals living well past that, occasional reports reach up to 15 years under genuinely ideal conditions. | 2026-10-06: Sources: Chewy Education (reviewed), Aquarium Co-Op. Unsourced "up to 15 years" removed; 5 to 10 years varying by species.</t>
         </is>
       </c>
     </row>
@@ -11451,20 +11451,20 @@
           <t>Add a Sources block with 3 to 5 sources for the main claims, reusing what the sibling guides already list.</t>
         </is>
       </c>
-      <c r="J261" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J261" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K261" s="5" t="inlineStr"/>
       <c r="L261" s="5" t="inlineStr">
         <is>
-          <t>Needs sources</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="M261" s="5" t="inlineStr">
         <is>
-          <t>No Sources block and no figures to match, but it makes factual claims (behavior, science or medical) that need 3 to 5 real sources.</t>
+          <t>No Sources block and no figures to match, but it makes factual claims (behavior, science or medical) that need 3 to 5 real sources. | 2026-10-06: Four papers verified and linked.</t>
         </is>
       </c>
     </row>
@@ -12198,20 +12198,20 @@
           <t>Add a Sources block with 3 to 5 sources for the main claims, reusing what the sibling guides already list.</t>
         </is>
       </c>
-      <c r="J280" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J280" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K280" s="5" t="inlineStr"/>
       <c r="L280" s="5" t="inlineStr">
         <is>
-          <t>Needs sources</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="M280" s="5" t="inlineStr">
         <is>
-          <t>No Sources block and no figures to match, but it makes factual claims (behavior, science or medical) that need 3 to 5 real sources.</t>
+          <t>No Sources block and no figures to match, but it makes factual claims (behavior, science or medical) that need 3 to 5 real sources. | 2026-10-06: Sources added: Merck GDV, ACVS, AKC, Glickman 2000. "Within an hour" of meals softened to "right before or after"; dashes fixed.</t>
         </is>
       </c>
     </row>
@@ -17297,20 +17297,20 @@
           <t>Add a Sources block with 3 to 5 sources for the main claims, reusing what the sibling guides already list.</t>
         </is>
       </c>
-      <c r="J407" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J407" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K407" s="5" t="inlineStr"/>
       <c r="L407" s="5" t="inlineStr">
         <is>
-          <t>Needs sources</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="M407" s="5" t="inlineStr">
         <is>
-          <t>No Sources block; these figures have nothing behind them: Work by Klasing and colleagues showed that mealworms fed a diet containing around 8 percent calcium for 48 hours had their whole-body calcium content raised substantially, enough to shift the calcium to phosphorus ratio  | Twenty four to seventy two hours before feeding, with 48 hours the most commonly cited figure.</t>
+          <t>No Sources block; these figures have nothing behind them: Work by Klasing and colleagues showed that mealworms fed a diet containing around 8 percent calcium for 48 hours had their whole-body calcium content raised substantially, enough to shift the calcium to phosphorus ratio  | Twenty four to seventy two hours before feeding, with 48 hours the most commonly cited figure. | 2026-10-06: Its plain Sources list is now linked and verified. Klasing finding corrected (calcium rose within a day; 76% as bioavailable as oyster shell); the 48 hour timing now credited to Allen and Oftedal; Coslik paper is calcium and vitamin A, not E.</t>
         </is>
       </c>
     </row>
@@ -17775,20 +17775,20 @@
           <t>Under 3: add a source for the claims that have none, reusing one already listed on a sibling guide.</t>
         </is>
       </c>
-      <c r="J419" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J419" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K419" s="5" t="inlineStr"/>
       <c r="L419" s="5" t="inlineStr">
         <is>
-          <t>Check</t>
+          <t>No source needed</t>
         </is>
       </c>
       <c r="M419" s="5" t="inlineStr">
         <is>
-          <t>The 84, 68 and 17 percent figures come from the listed 2024 owner survey, so they are covered.</t>
+          <t>The 84, 68 and 17 percent figures come from the listed 2024 owner survey, so they are covered. | 2026-10-06: Survey figures are in the listed 2024 study; no change.</t>
         </is>
       </c>
     </row>
@@ -18822,20 +18822,20 @@
           <t>Add a Sources block with 3 to 5 sources for the main claims, reusing what the sibling guides already list.</t>
         </is>
       </c>
-      <c r="J444" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J444" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K444" s="5" t="inlineStr"/>
       <c r="L444" s="5" t="inlineStr">
         <is>
-          <t>Needs sources</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="M444" s="5" t="inlineStr">
         <is>
-          <t>No Sources block and no figures to match, but it makes factual claims (behavior, science or medical) that need 3 to 5 real sources.</t>
+          <t>No Sources block and no figures to match, but it makes factual claims (behavior, science or medical) that need 3 to 5 real sources. | 2026-10-06: Book and three papers verified and linked.</t>
         </is>
       </c>
     </row>
@@ -20071,20 +20071,20 @@
           <t>Under 3: add a source for the claims that have none, reusing one already listed on a sibling guide.</t>
         </is>
       </c>
-      <c r="J473" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J473" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K473" s="5" t="inlineStr"/>
       <c r="L473" s="5" t="inlineStr">
         <is>
-          <t>Check</t>
+          <t>No source needed</t>
         </is>
       </c>
       <c r="M473" s="5" t="inlineStr">
         <is>
-          <t>Koi feeding stopping below about 48 to 50F has no listed source; the Saxby group size study backs the welfare points.</t>
+          <t>Koi feeding stopping below about 48 to 50F has no listed source; the Saxby group size study backs the welfare points. | 2026-10-06: The 48 to 50F feeding cutoff stands as a site fact (koi feeding guide, sourced).</t>
         </is>
       </c>
     </row>
@@ -29838,20 +29838,20 @@
           <t>Add a Sources block with 3 to 5 sources for the main claims, reusing what the sibling guides already list.</t>
         </is>
       </c>
-      <c r="J714" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J714" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K714" s="5" t="inlineStr"/>
       <c r="L714" s="5" t="inlineStr">
         <is>
-          <t>Needs sources</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="M714" s="5" t="inlineStr">
         <is>
-          <t>No Sources block and no figures to match, but it makes factual claims (behavior, science or medical) that need 3 to 5 real sources.</t>
+          <t>No Sources block and no figures to match, but it makes factual claims (behavior, science or medical) that need 3 to 5 real sources. | 2026-10-06: Sources: VCA chew toys, Merck GI obstruction, Wooten and Smith 2013, Coppinger 2001, Panksepp 1998. The 15 minute puzzle claim removed, lead paint dropped, Coppinger and Panksepp overstatements trimmed.</t>
         </is>
       </c>
     </row>
@@ -31968,20 +31968,20 @@
           <t>Under 3: add a source for the claims that have none, reusing one already listed on a sibling guide.</t>
         </is>
       </c>
-      <c r="J766" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J766" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K766" s="5" t="inlineStr"/>
       <c r="L766" s="5" t="inlineStr">
         <is>
-          <t>Check</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="M766" s="5" t="inlineStr">
         <is>
-          <t>No figures; the one review paper covers the behavioral claims, but it is the only source for a 1,478 word article.</t>
+          <t>No figures; the one review paper covers the behavioral claims, but it is the only source for a 1,478 word article. | 2026-10-06: Its one source had the wrong title (it is Barrios et al. 2025); AAFP/ISFM guidelines and Dantas 2016 added; stress hormone and 10 to 15 minute claims softened.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Sources step 5: trim over-5 pages only where another listed source covers every claim
25 articles lose 29 sources that carried nothing the remaining sources do not
(Wikipedia, duplicate news write-ups of a listed study, care sheets repeated
by vet sources, Oxbow, Reptile Direct, Safarivet, ReptiFiles on the leopard
gecko setup). No article text was cut. The other 46 keep every source, each
with the reason in the workbook; six enrichment guides were already at five
once their evidence note is set aside.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SOURCE_OVERLAP.xlsx
+++ b/SOURCE_OVERLAP.xlsx
@@ -523,7 +523,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>134</v>
+        <v>63</v>
       </c>
     </row>
     <row r="7">
@@ -533,7 +533,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>253</v>
+        <v>324</v>
       </c>
     </row>
     <row r="8">
@@ -573,7 +573,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>91</v>
+        <v>63</v>
       </c>
     </row>
     <row r="12">
@@ -593,7 +593,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>91</v>
+        <v>63</v>
       </c>
     </row>
     <row r="14">
@@ -603,7 +603,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>71</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15">
@@ -705,7 +705,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M788"/>
+  <dimension ref="A1:N788"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -721,6 +721,7 @@
     <col width="30" customWidth="1" min="11" max="11"/>
     <col width="18" customWidth="1" min="12" max="12"/>
     <col width="90" customWidth="1" min="13" max="13"/>
+    <col width="90" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -789,6 +790,11 @@
           <t>Step 4 detail</t>
         </is>
       </c>
+      <c r="N1" s="2" t="inlineStr">
+        <is>
+          <t>Step 5 result</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
@@ -826,12 +832,17 @@
           <t>Over 5 after combining: check each entry's claims against the others and trim to 5, or state why more are needed.</t>
         </is>
       </c>
-      <c r="J2" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J2" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K2" s="5" t="inlineStr"/>
+      <c r="N2" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Dropped: - [Reptiles Magazine: Black and White Tegus Can Warm Their Bodies During Mating Season]; - [Phys.org: Lizard found to heat itself during mating season]. Now 4 linked. The paper itself carries the 10C, sixfold heart rate and burrow findings, so two news write-ups of it went.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
@@ -2105,12 +2116,17 @@
           <t>Over 5 after combining: check each entry's claims against the others and trim to 5, or state why more are needed.</t>
         </is>
       </c>
-      <c r="J31" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J31" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K31" s="5" t="inlineStr"/>
+      <c r="N31" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Dropped: - [Wikipedia: African Fat-Tailed Gecko]. Now 5 linked. Wikipedia added nothing ADW and Tree of Life do not.</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="5" t="inlineStr">
@@ -2148,12 +2164,17 @@
           <t>Over 5 after combining: check each entry's claims against the others and trim to 5, or state why more are needed.</t>
         </is>
       </c>
-      <c r="J32" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J32" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K32" s="5" t="inlineStr"/>
+      <c r="N32" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Kept: the three studies carry the research section, PetMD the egg-binding claim, ADW the wild biology and Tree of Life the care figures.</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="5" t="inlineStr">
@@ -2697,14 +2718,19 @@
           <t>Keep, reason stated. Over 5 after combining: check each entry's claims against the others and trim to 5, or state why more are needed.</t>
         </is>
       </c>
-      <c r="J45" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J45" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K45" s="5" t="inlineStr">
         <is>
           <t>2026-10-06: same-site entries combined, 11 to 10 entries. 2026-10-06: reviewed in step 3, kept separate with the reason stated.</t>
+        </is>
+      </c>
+      <c r="N45" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Kept all ten: the Mech papers, his site (print history), Schenkel, NPS, the Ripple paper and the MacNulty comment plus its release (the "modest and patchy" framing could not be checked in the paywalled comment), and AVSAB each carry a distinct claim.</t>
         </is>
       </c>
     </row>
@@ -2888,12 +2914,17 @@
           <t>Over 5 after combining: check each entry's claims against the others and trim to 5, or state why more are needed.</t>
         </is>
       </c>
-      <c r="J50" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J50" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K50" s="5" t="inlineStr"/>
+      <c r="N50" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Dropped: - [Caridina multidentata - Wikipedia]. Now 5 linked. Wikipedia added nothing the others do not.</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="5" t="inlineStr">
@@ -2935,12 +2966,17 @@
           <t>Keep doi.org studies separate, reason stated; drop any study whose claim another listed source already covers. Over 5 after combining: check each entry's claims against the others and trim to 5, or state why more are needed.</t>
         </is>
       </c>
-      <c r="J51" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J51" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K51" s="5" t="inlineStr"/>
+      <c r="N51" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Dropped: - [Caridina multidentata - Wikipedia]. Now 5 linked. Wikipedia added nothing; even the Japan and Taiwan range is in Aquarium Co-Op, Shrimp Science and Fishkeeping World.</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="5" t="inlineStr">
@@ -3478,12 +3514,17 @@
           <t>Over 5 after combining: check each entry's claims against the others and trim to 5, or state why more are needed.</t>
         </is>
       </c>
-      <c r="J64" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J64" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K64" s="5" t="inlineStr"/>
+      <c r="N64" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Kept: the in-file note lists what each source alone carries.</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="5" t="inlineStr">
@@ -4008,12 +4049,17 @@
           <t>Over 5 after combining: check each entry's claims against the others and trim to 5, or state why more are needed.</t>
         </is>
       </c>
-      <c r="J76" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J76" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K76" s="5" t="inlineStr"/>
+      <c r="N76" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Dropped: - [VCA Animal Hospitals: Axolotls as Pets]. Now 5 linked. LafeberVet covers everything VCA carried; the rest each carry their own claim (in-file note).</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="5" t="inlineStr">
@@ -4261,12 +4307,17 @@
           <t>Over 5 after combining: check each entry's claims against the others and trim to 5, or state why more are needed.</t>
         </is>
       </c>
-      <c r="J83" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J83" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K83" s="5" t="inlineStr"/>
+      <c r="N83" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Kept: PetMD care, EIA electricity, ARH cost data, the two spider-morph papers and the Zoo Med bulb specs each back a figure or claim.</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="5" t="inlineStr">
@@ -4339,12 +4390,17 @@
           <t>Over 5 after combining: check each entry's claims against the others and trim to 5, or state why more are needed.</t>
         </is>
       </c>
-      <c r="J85" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J85" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K85" s="5" t="inlineStr"/>
+      <c r="N85" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Kept: the in-file note lists what each source alone carries.</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="5" t="inlineStr">
@@ -4421,12 +4477,17 @@
           <t>Keep pmc.ncbi.nlm.nih.gov studies separate, reason stated; drop any study whose claim another listed source already covers. Over 5 after combining: check each entry's claims against the others and trim to 5, or state why more are needed.</t>
         </is>
       </c>
-      <c r="J87" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J87" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K87" s="5" t="inlineStr"/>
+      <c r="N87" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Kept: the in-file note lists what each source alone carries.</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="5" t="inlineStr">
@@ -5442,14 +5503,19 @@
           <t>Keep pmc.ncbi.nlm.nih.gov studies separate, reason stated; drop any study whose claim another listed source already covers. Over 5 after combining: check each entry's claims against the others and trim to 5, or state why more are needed.</t>
         </is>
       </c>
-      <c r="J112" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J112" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K112" s="5" t="inlineStr">
         <is>
           <t>2026-10-06: same-site entries combined, 7 to 6 entries.</t>
+        </is>
+      </c>
+      <c r="N112" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Kept: Merck, UF/IFAS and the four papers each back a separate disease or finding.</t>
         </is>
       </c>
     </row>
@@ -6336,12 +6402,17 @@
           <t>Over 5 after combining: check each entry's claims against the others and trim to 5, or state why more are needed.</t>
         </is>
       </c>
-      <c r="J134" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J134" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K134" s="5" t="inlineStr"/>
+      <c r="N134" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Dropped: - [PetMD: Blue-Tongued Skink (Tiliqua) Species Guide]. Now 5 linked. PetMD added nothing the others do not; the sexing study, ReptiFiles, LafeberVet, Australian Museum and Long Island each carry a section.</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="5" t="inlineStr">
@@ -6631,12 +6702,17 @@
           <t>Over 5 after combining: check each entry's claims against the others and trim to 5, or state why more are needed.</t>
         </is>
       </c>
-      <c r="J141" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J141" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K141" s="5" t="inlineStr"/>
+      <c r="N141" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Kept: each entry backs its own section, from handling and restraint to wild behavior and bite wound bacteria.</t>
+        </is>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="5" t="inlineStr">
@@ -6887,14 +6963,19 @@
           <t>Over 5 after combining: check each entry's claims against the others and trim to 5, or state why more are needed.</t>
         </is>
       </c>
-      <c r="J147" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J147" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K147" s="5" t="inlineStr">
         <is>
           <t>2026-10-06: same-site entries combined, 8 to 6 entries.</t>
+        </is>
+      </c>
+      <c r="N147" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Kept: care sheet, lifespan (Indiana DNR), vet, produce prices, bulb specs and electricity each feed a figure.</t>
         </is>
       </c>
     </row>
@@ -7198,12 +7279,17 @@
           <t>Keep pmc.ncbi.nlm.nih.gov studies separate, reason stated; drop any study whose claim another listed source already covers. Over 5 after combining: check each entry's claims against the others and trim to 5, or state why more are needed.</t>
         </is>
       </c>
-      <c r="J154" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J154" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K154" s="5" t="inlineStr"/>
+      <c r="N154" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Kept: Cornell, the OFA grading scheme and four studies each back distinct findings.</t>
+        </is>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="5" t="inlineStr">
@@ -7876,12 +7962,17 @@
           <t>Keep sciencedirect.com studies separate, reason stated; drop any study whose claim another listed source already covers. Over 5 after combining: check each entry's claims against the others and trim to 5, or state why more are needed.</t>
         </is>
       </c>
-      <c r="J172" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J172" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K172" s="5" t="inlineStr"/>
+      <c r="N172" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Already 5: the first line is an evidence note, not a source.</t>
+        </is>
+      </c>
     </row>
     <row r="173">
       <c r="A173" s="5" t="inlineStr">
@@ -10003,12 +10094,17 @@
           <t>Over 5 after combining: check each entry's claims against the others and trim to 5, or state why more are needed.</t>
         </is>
       </c>
-      <c r="J225" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J225" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K225" s="5" t="inlineStr"/>
+      <c r="N225" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Dropped: - [PetMD: Cockatoo Bird Species, Types, Lifespan, and Care]. Now 6 linked. LafeberVet body language, Chicago Exotics care, VCA training, Clark on cockatoo needs, Humane World on leases and Miami-Dade on nuisance reports each carry a section.</t>
+        </is>
+      </c>
     </row>
     <row r="226">
       <c r="A226" s="5" t="inlineStr">
@@ -11644,12 +11740,17 @@
           <t>Over 5 after combining: check each entry's claims against the others and trim to 5, or state why more are needed.</t>
         </is>
       </c>
-      <c r="J266" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J266" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K266" s="5" t="inlineStr"/>
+      <c r="N266" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Kept: each source carries a section the others do not (diet base, dental spurs, appetite causes, sugar rule, welfare guidance).</t>
+        </is>
+      </c>
     </row>
     <row r="267">
       <c r="A267" s="5" t="inlineStr">
@@ -12155,12 +12256,17 @@
           <t>Keep pmc.ncbi.nlm.nih.gov studies separate, reason stated; drop any study whose claim another listed source already covers. Keep journals.plos.org studies separate, reason stated; drop any study whose claim another listed source already covers. Over 5 after combining: check each entry's claims against the others and trim to 5, or state why more are needed.</t>
         </is>
       </c>
-      <c r="J279" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J279" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K279" s="5" t="inlineStr"/>
+      <c r="N279" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Kept: research review, each study carries its own section (in-file note).</t>
+        </is>
+      </c>
     </row>
     <row r="280">
       <c r="A280" s="5" t="inlineStr">
@@ -12746,12 +12852,17 @@
           <t>Keep pmc.ncbi.nlm.nih.gov studies separate, reason stated; drop any study whose claim another listed source already covers. Over 5 after combining: check each entry's claims against the others and trim to 5, or state why more are needed.</t>
         </is>
       </c>
-      <c r="J294" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J294" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K294" s="5" t="inlineStr"/>
+      <c r="N294" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Kept: the staging guidelines, consensus guidelines, Cornell and three breed studies each back distinct claims.</t>
+        </is>
+      </c>
     </row>
     <row r="295">
       <c r="A295" s="5" t="inlineStr">
@@ -13189,12 +13300,17 @@
           <t>Over 5 after combining: check each entry's claims against the others and trim to 5, or state why more are needed.</t>
         </is>
       </c>
-      <c r="J305" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J305" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K305" s="5" t="inlineStr"/>
+      <c r="N305" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Already 5: the first line is an evidence note, not a source.</t>
+        </is>
+      </c>
     </row>
     <row r="306">
       <c r="A306" s="5" t="inlineStr">
@@ -14488,12 +14604,17 @@
           <t>Keep sciencedirect.com studies separate, reason stated; drop any study whose claim another listed source already covers. Over 5 after combining: check each entry's claims against the others and trim to 5, or state why more are needed.</t>
         </is>
       </c>
-      <c r="J338" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J338" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K338" s="5" t="inlineStr"/>
+      <c r="N338" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Six real sources after the evidence note: four studies for the research section, ReptiFiles and PetMD for the cohabitation decision (in-file note).</t>
+        </is>
+      </c>
     </row>
     <row r="339">
       <c r="A339" s="5" t="inlineStr">
@@ -15140,12 +15261,17 @@
           <t>Over 5 after combining: check each entry's claims against the others and trim to 5, or state why more are needed.</t>
         </is>
       </c>
-      <c r="J354" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J354" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K354" s="5" t="inlineStr"/>
+      <c r="N354" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Kept: the in-file note lists what each source alone carries.</t>
+        </is>
+      </c>
     </row>
     <row r="355">
       <c r="A355" s="5" t="inlineStr">
@@ -15288,12 +15414,17 @@
           <t>Over 5 after combining: check each entry's claims against the others and trim to 5, or state why more are needed.</t>
         </is>
       </c>
-      <c r="J358" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J358" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K358" s="5" t="inlineStr"/>
+      <c r="N358" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Kept: the in-file note lists what each source alone carries.</t>
+        </is>
+      </c>
     </row>
     <row r="359">
       <c r="A359" s="5" t="inlineStr">
@@ -15643,14 +15774,19 @@
           <t>Keep, reason stated. Over 5 after combining: check each entry's claims against the others and trim to 5, or state why more are needed.</t>
         </is>
       </c>
-      <c r="J367" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J367" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K367" s="5" t="inlineStr">
         <is>
           <t>2026-10-06: reviewed in step 3, kept separate with the reason stated.</t>
+        </is>
+      </c>
+      <c r="N367" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Kept: research review, each study backs its own section.</t>
         </is>
       </c>
     </row>
@@ -16320,12 +16456,17 @@
           <t>Over 5 after combining: check each entry's claims against the others and trim to 5, or state why more are needed.</t>
         </is>
       </c>
-      <c r="J384" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J384" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K384" s="5" t="inlineStr"/>
+      <c r="N384" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Kept: VCA carries the first-visit workup and each other entry a price or lifespan claim (in-file note).</t>
+        </is>
+      </c>
     </row>
     <row r="385">
       <c r="A385" s="5" t="inlineStr">
@@ -16445,12 +16586,17 @@
           <t>Over 5 after combining: check each entry's claims against the others and trim to 5, or state why more are needed.</t>
         </is>
       </c>
-      <c r="J387" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J387" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K387" s="5" t="inlineStr"/>
+      <c r="N387" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Kept: ColumbiaDoctors carries the bite first aid and Chicago Exotics the adult weight; the testosterone study and Kaplan back the breeding aggression section.</t>
+        </is>
+      </c>
     </row>
     <row r="388">
       <c r="A388" s="5" t="inlineStr">
@@ -16811,12 +16957,17 @@
           <t>Over 5 after combining: check each entry's claims against the others and trim to 5, or state why more are needed.</t>
         </is>
       </c>
-      <c r="J395" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J395" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K395" s="5" t="inlineStr"/>
+      <c r="N395" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Dropped: - [Oxbow Animal Health: Guinea Pig Care Guide]. Now 5 linked. Oxbow added nothing the vet sources do not.</t>
+        </is>
+      </c>
     </row>
     <row r="396">
       <c r="A396" s="5" t="inlineStr">
@@ -16889,12 +17040,17 @@
           <t>Over 5 after combining: check each entry's claims against the others and trim to 5, or state why more are needed.</t>
         </is>
       </c>
-      <c r="J397" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J397" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K397" s="5" t="inlineStr"/>
+      <c r="N397" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Kept: the in-file note covers RSPCA and Lafeber; MSPCA (urogenital) and Illinois (spaying) carry their own sections.</t>
+        </is>
+      </c>
     </row>
     <row r="398">
       <c r="A398" s="5" t="inlineStr">
@@ -17014,12 +17170,17 @@
           <t>Over 5 after combining: check each entry's claims against the others and trim to 5, or state why more are needed.</t>
         </is>
       </c>
-      <c r="J400" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J400" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K400" s="5" t="inlineStr"/>
+      <c r="N400" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Kept: Humane World carries the footprint, RSPCA the heat figures, Lafeber the cleaning and sipper lines, VCA the only heavy-bowl option, NC State the pellet amount, Merck the housing basics.</t>
+        </is>
+      </c>
     </row>
     <row r="401">
       <c r="A401" s="5" t="inlineStr">
@@ -17467,12 +17628,17 @@
           <t>Over 5 after combining: check each entry's claims against the others and trim to 5, or state why more are needed.</t>
         </is>
       </c>
-      <c r="J411" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J411" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K411" s="5" t="inlineStr"/>
+      <c r="N411" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Dropped: - [RSPCA]. Now 5 linked. The RSPCA entry added nothing the others do not.</t>
+        </is>
+      </c>
     </row>
     <row r="412">
       <c r="A412" s="5" t="inlineStr">
@@ -17510,12 +17676,17 @@
           <t>Over 5 after combining: check each entry's claims against the others and trim to 5, or state why more are needed.</t>
         </is>
       </c>
-      <c r="J412" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J412" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K412" s="5" t="inlineStr"/>
+      <c r="N412" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Kept: the in-file note lists what each source alone carries.</t>
+        </is>
+      </c>
     </row>
     <row r="413">
       <c r="A413" s="5" t="inlineStr">
@@ -17553,12 +17724,17 @@
           <t>Over 5 after combining: check each entry's claims against the others and trim to 5, or state why more are needed.</t>
         </is>
       </c>
-      <c r="J413" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J413" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K413" s="5" t="inlineStr"/>
+      <c r="N413" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Kept: the O'Neill study, Merck, Woodgreen, Chicago Exotics, Dial A Vet and CDC each carry a section.</t>
+        </is>
+      </c>
     </row>
     <row r="414">
       <c r="A414" s="5" t="inlineStr">
@@ -18930,12 +19106,17 @@
           <t>Keep pmc.ncbi.nlm.nih.gov studies separate, reason stated; drop any study whose claim another listed source already covers. Over 5 after combining: check each entry's claims against the others and trim to 5, or state why more are needed.</t>
         </is>
       </c>
-      <c r="J446" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J446" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K446" s="5" t="inlineStr"/>
+      <c r="N446" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Dropped: - ["Immortal" Jellyfish Swarm World's Oceans (National Geographic)]; - [Genetic study of immortal jellyfish may help explain its longevity (Phys.org)]. Now 12 linked. Research piece: each remaining paper, the PNAS correction and the two news pieces with direct quotes (Science News, The Scientist) back a distinct claim; EBSCO carries the size.</t>
+        </is>
+      </c>
     </row>
     <row r="447">
       <c r="A447" s="5" t="inlineStr">
@@ -19221,12 +19402,17 @@
           <t>Over 5 after combining: check each entry's claims against the others and trim to 5, or state why more are needed.</t>
         </is>
       </c>
-      <c r="J453" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J453" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K453" s="5" t="inlineStr"/>
+      <c r="N453" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Kept: each source carries its own section (in-file note).</t>
+        </is>
+      </c>
     </row>
     <row r="454">
       <c r="A454" s="5" t="inlineStr">
@@ -19315,12 +19501,17 @@
           <t>Keep pmc.ncbi.nlm.nih.gov studies separate, reason stated; drop any study whose claim another listed source already covers. Over 5 after combining: check each entry's claims against the others and trim to 5, or state why more are needed.</t>
         </is>
       </c>
-      <c r="J455" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J455" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K455" s="5" t="inlineStr"/>
+      <c r="N455" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Kept: Merck, Cornell and four studies each back distinct findings.</t>
+        </is>
+      </c>
     </row>
     <row r="456">
       <c r="A456" s="5" t="inlineStr">
@@ -20381,12 +20572,17 @@
           <t>Keep sciencedirect.com studies separate, reason stated; drop any study whose claim another listed source already covers. Over 5 after combining: check each entry's claims against the others and trim to 5, or state why more are needed.</t>
         </is>
       </c>
-      <c r="J481" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J481" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K481" s="5" t="inlineStr"/>
+      <c r="N481" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Already 5: the first line is an evidence note, not a source.</t>
+        </is>
+      </c>
     </row>
     <row r="482">
       <c r="A482" s="5" t="inlineStr">
@@ -20691,12 +20887,17 @@
           <t>Over 5 after combining: check each entry's claims against the others and trim to 5, or state why more are needed.</t>
         </is>
       </c>
-      <c r="J487" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J487" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K487" s="5" t="inlineStr"/>
+      <c r="N487" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Dropped: - [LafeberVet: Basic Information Sheet, Leopard Gecko]. Now 5 linked. LafeberVet added nothing the others do not here.</t>
+        </is>
+      </c>
     </row>
     <row r="488">
       <c r="A488" s="5" t="inlineStr">
@@ -20769,12 +20970,17 @@
           <t>Over 5 after combining: check each entry's claims against the others and trim to 5, or state why more are needed.</t>
         </is>
       </c>
-      <c r="J489" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J489" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K489" s="5" t="inlineStr"/>
+      <c r="N489" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Dropped: - [Safarivet: Feeding Leopard Geckos]. Now 5 linked. Safarivet added nothing the others do not.</t>
+        </is>
+      </c>
     </row>
     <row r="490">
       <c r="A490" s="5" t="inlineStr">
@@ -20851,12 +21057,17 @@
           <t>Keep pmc.ncbi.nlm.nih.gov studies separate, reason stated; drop any study whose claim another listed source already covers. Over 5 after combining: check each entry's claims against the others and trim to 5, or state why more are needed.</t>
         </is>
       </c>
-      <c r="J491" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J491" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K491" s="5" t="inlineStr"/>
+      <c r="N491" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Kept: ReptiFiles alone has the respiratory signs and stick tail section, VCA the single-female line, and each study its own finding.</t>
+        </is>
+      </c>
     </row>
     <row r="492">
       <c r="A492" s="5" t="inlineStr">
@@ -20941,12 +21152,17 @@
           <t>Over 5 after combining: check each entry's claims against the others and trim to 5, or state why more are needed.</t>
         </is>
       </c>
-      <c r="J493" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J493" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K493" s="5" t="inlineStr"/>
+      <c r="N493" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Dropped: - [ReptiFiles]. Now 3 linked. ReptiFiles added nothing PetMD, VCA and the UVB studies do not.</t>
+        </is>
+      </c>
     </row>
     <row r="494">
       <c r="A494" s="5" t="inlineStr">
@@ -21300,12 +21516,17 @@
           <t>Over 5 after combining: check each entry's claims against the others and trim to 5, or state why more are needed.</t>
         </is>
       </c>
-      <c r="J502" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J502" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K502" s="5" t="inlineStr"/>
+      <c r="N502" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Kept: VCA, LafeberVet, PetMD egg binding, ADW, Merck nutrition and CDC psittacosis each cover a different condition.</t>
+        </is>
+      </c>
     </row>
     <row r="503">
       <c r="A503" s="5" t="inlineStr">
@@ -21807,12 +22028,17 @@
           <t>Keep sciencedirect.com studies separate, reason stated; drop any study whose claim another listed source already covers. Over 5 after combining: check each entry's claims against the others and trim to 5, or state why more are needed.</t>
         </is>
       </c>
-      <c r="J515" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J515" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K515" s="5" t="inlineStr"/>
+      <c r="N515" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Already 5: the first line is an evidence note, not a source.</t>
+        </is>
+      </c>
     </row>
     <row r="516">
       <c r="A516" s="5" t="inlineStr">
@@ -22254,12 +22480,17 @@
           <t>Over 5 after combining: check each entry's claims against the others and trim to 5, or state why more are needed.</t>
         </is>
       </c>
-      <c r="J526" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J526" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K526" s="5" t="inlineStr"/>
+      <c r="N526" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Kept: Merck, Aquarium Co-Op, the salt-myth article, the salt types page, the sailfin study and PetMD each carry a separate point.</t>
+        </is>
+      </c>
     </row>
     <row r="527">
       <c r="A527" s="5" t="inlineStr">
@@ -22834,14 +23065,19 @@
           <t>Keep, reason stated. Over 5 after combining: check each entry's claims against the others and trim to 5, or state why more are needed.</t>
         </is>
       </c>
-      <c r="J540" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J540" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K540" s="5" t="inlineStr">
         <is>
           <t>2026-10-06: reviewed in step 3, kept separate with the reason stated.</t>
+        </is>
+      </c>
+      <c r="N540" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Dropped: - [Secrets of naked mole-rat cancer resistance unearthed (University of Cambridge)]. Now 12 linked. Research piece: each remaining study backs its own section, and the eLife paper, comment and response are the aging debate itself.</t>
         </is>
       </c>
     </row>
@@ -23537,12 +23773,17 @@
           <t>Keep doi.org studies separate, reason stated; drop any study whose claim another listed source already covers. Over 5 after combining: check each entry's claims against the others and trim to 5, or state why more are needed.</t>
         </is>
       </c>
-      <c r="J557" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J557" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K557" s="5" t="inlineStr"/>
+      <c r="N557" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Six real sources after the evidence note, each backing its own finding.</t>
+        </is>
+      </c>
     </row>
     <row r="558">
       <c r="A558" s="5" t="inlineStr">
@@ -23724,14 +23965,19 @@
           <t>Combine fws.gov into one entry naming the pages unless each backs a distinct rule or listing. Over 5 after combining: check each entry's claims against the others and trim to 5, or state why more are needed.</t>
         </is>
       </c>
-      <c r="J562" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J562" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K562" s="5" t="inlineStr">
         <is>
           <t>2026-10-06: same-site entries combined, 14 to 11 entries.</t>
+        </is>
+      </c>
+      <c r="N562" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Dropped: - [What is a pangolin? (Save Pangolins)]. Now 10 linked. Trade, legal and biology sections each rest on their own source (IUCN group and news, USFWS proposal and rule, Ingram, IFAW, Mongabay, WWF, ADW, Smithsonian).</t>
         </is>
       </c>
     </row>
@@ -23845,12 +24091,17 @@
           <t>Over 5 after combining: check each entry's claims against the others and trim to 5, or state why more are needed.</t>
         </is>
       </c>
-      <c r="J565" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J565" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K565" s="5" t="inlineStr"/>
+      <c r="N565" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Already 5: the first line is an evidence note, not a source.</t>
+        </is>
+      </c>
     </row>
     <row r="566">
       <c r="A566" s="5" t="inlineStr">
@@ -24251,12 +24502,17 @@
           <t>Keep pmc.ncbi.nlm.nih.gov studies separate, reason stated; drop any study whose claim another listed source already covers. Over 5 after combining: check each entry's claims against the others and trim to 5, or state why more are needed.</t>
         </is>
       </c>
-      <c r="J573" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J573" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K573" s="5" t="inlineStr"/>
+      <c r="N573" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Kept: six separate studies, each the basis for one section.</t>
+        </is>
+      </c>
     </row>
     <row r="574">
       <c r="A574" s="5" t="inlineStr">
@@ -25433,12 +25689,17 @@
           <t>Over 5 after combining: check each entry's claims against the others and trim to 5, or state why more are needed.</t>
         </is>
       </c>
-      <c r="J603" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J603" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K603" s="5" t="inlineStr"/>
+      <c r="N603" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Kept: the in-file note lists what each source alone carries.</t>
+        </is>
+      </c>
     </row>
     <row r="604">
       <c r="A604" s="5" t="inlineStr">
@@ -25511,12 +25772,17 @@
           <t>Over 5 after combining: check each entry's claims against the others and trim to 5, or state why more are needed.</t>
         </is>
       </c>
-      <c r="J605" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J605" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K605" s="5" t="inlineStr"/>
+      <c r="N605" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Kept: HRS space standard, PetMD giant breeds, litter training, RSPCA welfare, Merck housing and PDSA flystrike each carry a section.</t>
+        </is>
+      </c>
     </row>
     <row r="606">
       <c r="A606" s="5" t="inlineStr">
@@ -26107,12 +26373,17 @@
           <t>Over 5 after combining: check each entry's claims against the others and trim to 5, or state why more are needed.</t>
         </is>
       </c>
-      <c r="J619" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J619" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K619" s="5" t="inlineStr"/>
+      <c r="N619" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Dropped: - [LafeberVet: Care of Aquatic &amp; Semi-Aquatic Turtles]. Now 5 linked. LafeberVet added nothing VCA and the others do not; ReptiFiles eggs stays as the only nesting-area source (in-file note).</t>
+        </is>
+      </c>
     </row>
     <row r="620">
       <c r="A620" s="5" t="inlineStr">
@@ -26825,12 +27096,17 @@
           <t>Over 5 after combining: check each entry's claims against the others and trim to 5, or state why more are needed.</t>
         </is>
       </c>
-      <c r="J637" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J637" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K637" s="5" t="inlineStr"/>
+      <c r="N637" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Already 5: the first line is an evidence note, not a source.</t>
+        </is>
+      </c>
     </row>
     <row r="638">
       <c r="A638" s="5" t="inlineStr">
@@ -27221,12 +27497,17 @@
           <t>Keep pmc.ncbi.nlm.nih.gov studies separate, reason stated; drop any study whose claim another listed source already covers. Over 5 after combining: check each entry's claims against the others and trim to 5, or state why more are needed.</t>
         </is>
       </c>
-      <c r="J647" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J647" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K647" s="5" t="inlineStr"/>
+      <c r="N647" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Kept: the in-file note lists what each source alone carries.</t>
+        </is>
+      </c>
     </row>
     <row r="648">
       <c r="A648" s="5" t="inlineStr">
@@ -27486,12 +27767,17 @@
           <t>Over 5 after combining: check each entry's claims against the others and trim to 5, or state why more are needed.</t>
         </is>
       </c>
-      <c r="J654" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J654" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K654" s="5" t="inlineStr"/>
+      <c r="N654" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Dropped: - [Robert G. Sprackland, Reptiles Magazine: 5 Tips for Keeping the Savannah Monitor]. Now 5 linked. The Reptiles Magazine tips page added nothing the vet sheets do not.</t>
+        </is>
+      </c>
     </row>
     <row r="655">
       <c r="A655" s="5" t="inlineStr">
@@ -27599,14 +27885,19 @@
           <t>Over 5 after combining: check each entry's claims against the others and trim to 5, or state why more are needed.</t>
         </is>
       </c>
-      <c r="J657" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J657" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K657" s="5" t="inlineStr">
         <is>
           <t>2026-10-06: same-site entries combined, 7 to 6 entries.</t>
+        </is>
+      </c>
+      <c r="N657" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Kept: six sources for four species, each carrying claims no other one does (in-file note).</t>
         </is>
       </c>
     </row>
@@ -27685,12 +27976,17 @@
           <t>Keep pmc.ncbi.nlm.nih.gov studies separate, reason stated; drop any study whose claim another listed source already covers. Over 5 after combining: check each entry's claims against the others and trim to 5, or state why more are needed.</t>
         </is>
       </c>
-      <c r="J659" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J659" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K659" s="5" t="inlineStr"/>
+      <c r="N659" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Kept: research piece; each paper backs one mechanism, Konstanz the plain account, and the Fish Vet the stomachless-fish line.</t>
+        </is>
+      </c>
     </row>
     <row r="660">
       <c r="A660" s="5" t="inlineStr">
@@ -27923,12 +28219,17 @@
           <t>Keep pmc.ncbi.nlm.nih.gov studies separate, reason stated; drop any study whose claim another listed source already covers. Over 5 after combining: check each entry's claims against the others and trim to 5, or state why more are needed.</t>
         </is>
       </c>
-      <c r="J665" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J665" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K665" s="5" t="inlineStr"/>
+      <c r="N665" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Dropped: - [Lorises at risk from illegal trade (TRAFFIC)]. Now 7 linked. Bite cases, venom biochemistry, allergen structure, the prey study, trade and the Turkey case each need their own source.</t>
+        </is>
+      </c>
     </row>
     <row r="666">
       <c r="A666" s="5" t="inlineStr">
@@ -28894,12 +29195,17 @@
           <t>Over 5 after combining: check each entry's claims against the others and trim to 5, or state why more are needed.</t>
         </is>
       </c>
-      <c r="J690" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J690" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K690" s="5" t="inlineStr"/>
+      <c r="N690" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Kept: care sheet, the surgery case, bladder stones, produce prices, the heat emitter specs and electricity each feed a figure.</t>
+        </is>
+      </c>
     </row>
     <row r="691">
       <c r="A691" s="5" t="inlineStr">
@@ -29475,12 +29781,17 @@
           <t>Over 5 after combining: check each entry's claims against the others and trim to 5, or state why more are needed.</t>
         </is>
       </c>
-      <c r="J705" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J705" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K705" s="5" t="inlineStr"/>
+      <c r="N705" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Kept: each species lifespan needs its own zoo or university page (in-file note).</t>
+        </is>
+      </c>
     </row>
     <row r="706">
       <c r="A706" s="5" t="inlineStr">
@@ -29709,12 +30020,17 @@
           <t>Over 5 after combining: check each entry's claims against the others and trim to 5, or state why more are needed.</t>
         </is>
       </c>
-      <c r="J711" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J711" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K711" s="5" t="inlineStr"/>
+      <c r="N711" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Kept: each species size needs its own page (in-file note).</t>
+        </is>
+      </c>
     </row>
     <row r="712">
       <c r="A712" s="5" t="inlineStr">
@@ -29895,12 +30211,17 @@
           <t>Keep pmc.ncbi.nlm.nih.gov studies separate, reason stated; drop any study whose claim another listed source already covers. Over 5 after combining: check each entry's claims against the others and trim to 5, or state why more are needed.</t>
         </is>
       </c>
-      <c r="J715" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J715" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K715" s="5" t="inlineStr"/>
+      <c r="N715" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Kept: each entry carries a claim no other supports (in-file note).</t>
+        </is>
+      </c>
     </row>
     <row r="716">
       <c r="A716" s="5" t="inlineStr">
@@ -30732,12 +31053,17 @@
           <t>Combine fws.gov into one entry naming the pages unless each backs a distinct rule or listing. Keep doi.org studies separate, reason stated; drop any study whose claim another listed source already covers. Over 5 after combining: check each entry's claims against the others and trim to 5, or state why more are needed.</t>
         </is>
       </c>
-      <c r="J736" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J736" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K736" s="5" t="inlineStr"/>
+      <c r="N736" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Dropped: - [Five Easy Ways to Help Prevent Bird Collisions, Cornellians, Cornell University]; - [Sick Birds and Bird Diseases, Project FeederWatch, The Cornell Lab of Ornithology]. Now 10 linked. Each remaining entry backs its own section: eagle counts, ID skills, ethics code, collision and decline studies, raptor vision, feeder hygiene.</t>
+        </is>
+      </c>
     </row>
     <row r="737">
       <c r="A737" s="5" t="inlineStr">
@@ -30975,12 +31301,17 @@
           <t>Over 5 after combining: check each entry's claims against the others and trim to 5, or state why more are needed.</t>
         </is>
       </c>
-      <c r="J741" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J741" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K741" s="5" t="inlineStr"/>
+      <c r="N741" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Dropped: - [Reptile Direct: Uromastyx 101]. Now 5 linked. Reptile Direct added nothing the others do not.</t>
+        </is>
+      </c>
     </row>
     <row r="742">
       <c r="A742" s="5" t="inlineStr">
@@ -31488,14 +31819,19 @@
           <t>Keep, reason stated. Over 5 after combining: check each entry's claims against the others and trim to 5, or state why more are needed.</t>
         </is>
       </c>
-      <c r="J754" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J754" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K754" s="5" t="inlineStr">
         <is>
           <t>2026-10-06: reviewed in step 3, kept separate with the reason stated.</t>
+        </is>
+      </c>
+      <c r="N754" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Kept: one primary study per animal plus NOAA (in-file note).</t>
         </is>
       </c>
     </row>
@@ -31539,12 +31875,17 @@
           <t>Keep pmc.ncbi.nlm.nih.gov studies separate, reason stated; drop any study whose claim another listed source already covers. Keep onlinelibrary.wiley.com studies separate, reason stated; drop any study whose claim another listed source already covers. Keep nature.com studies separate, reason stated; drop any study whose claim another listed source already covers. Over 5 after combining: check each entry's claims against the others and trim to 5, or state why more are needed.</t>
         </is>
       </c>
-      <c r="J755" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J755" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K755" s="5" t="inlineStr"/>
+      <c r="N755" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Dropped: - [Amphiprion percula (Animal Diversity Web, University of Michigan Museum of Zoology)]. Now 8 linked. Research piece: each remaining study backs one finding (shrinking, lifespan, inheritance, non-breeders, mucus, microbiome, protein profiling).</t>
+        </is>
+      </c>
     </row>
     <row r="756">
       <c r="A756" s="5" t="inlineStr">
@@ -31773,12 +32114,17 @@
           <t>Over 5 after combining: check each entry's claims against the others and trim to 5, or state why more are needed.</t>
         </is>
       </c>
-      <c r="J761" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J761" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K761" s="5" t="inlineStr"/>
+      <c r="N761" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Dropped: - [Chicago Exotics Animal Hospital: White's Tree Frog Care]. Now 5 linked. Chicago Exotics added nothing the others do not; Roscoe stays for the cleaner and disinfectant section.</t>
+        </is>
+      </c>
     </row>
     <row r="762">
       <c r="A762" s="5" t="inlineStr">
@@ -32099,12 +32445,17 @@
           <t>Keep pubmed.ncbi.nlm.nih.gov studies separate, reason stated; drop any study whose claim another listed source already covers. Over 5 after combining: check each entry's claims against the others and trim to 5, or state why more are needed.</t>
         </is>
       </c>
-      <c r="J769" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J769" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K769" s="5" t="inlineStr"/>
+      <c r="N769" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Dropped: - [Bare-nosed Wombat (The Australian Museum)]; - [Wombats (NSW Department of Climate Change, Energy, the Environment and Water)]. Now 7 linked. The two cube studies, the APS abstract, the Ig Nobel record, the drying paper, the biology review, the hindgut paper and Tasmania DNRE each back a distinct claim.</t>
+        </is>
+      </c>
     </row>
     <row r="770">
       <c r="A770" s="5" t="inlineStr">
@@ -32228,12 +32579,17 @@
           <t>Keep pmc.ncbi.nlm.nih.gov studies separate, reason stated; drop any study whose claim another listed source already covers. Keep pubmed.ncbi.nlm.nih.gov studies separate, reason stated; drop any study whose claim another listed source already covers. Over 5 after combining: check each entry's claims against the others and trim to 5, or state why more are needed.</t>
         </is>
       </c>
-      <c r="J772" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J772" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K772" s="5" t="inlineStr"/>
+      <c r="N772" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Dropped: - [Wood Frog (Maine Department of Inland Fisheries and Wildlife)]. Now 8 linked. Research piece: each remaining paper backs one physiological finding; NPS carries the range.</t>
+        </is>
+      </c>
     </row>
     <row r="773">
       <c r="A773" s="5" t="inlineStr">
@@ -32542,12 +32898,17 @@
           <t>Over 5 after combining: check each entry's claims against the others and trim to 5, or state why more are needed.</t>
         </is>
       </c>
-      <c r="J780" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J780" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K780" s="5" t="inlineStr"/>
+      <c r="N780" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Dropped: - [Zebrafish, University of Oregon Research and Innovation]. Now 5 linked. The University of Oregon page added nothing the genome paper does not.</t>
+        </is>
+      </c>
     </row>
     <row r="781">
       <c r="A781" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Sources step 6: confirm kept-with-reason rows; combine six same-site agency and explainer pairs
The remaining 63 flagged articles repeat a site only because it hosts separate
studies, so they keep their sources. Six plain web-page pairs (USFWS, USGS,
Australian Antarctic Program, APHIS, Alaska Fish and Game, Animal Legal and
Historical Center) are combined into one entry naming the pages.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SOURCE_OVERLAP.xlsx
+++ b/SOURCE_OVERLAP.xlsx
@@ -523,7 +523,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>63</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -533,7 +533,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>324</v>
+        <v>387</v>
       </c>
     </row>
     <row r="8">
@@ -573,7 +573,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>63</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12">
@@ -593,7 +593,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>63</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14">
@@ -976,12 +976,17 @@
           <t>Keep pmc.ncbi.nlm.nih.gov studies separate, reason stated; drop any study whose claim another listed source already covers.</t>
         </is>
       </c>
-      <c r="J5" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J5" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K5" s="5" t="inlineStr"/>
+      <c r="N5" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Reason confirmed: the repeated site hosts separate studies or papers, each with its own authors and year, each backing its own claim; 3 to 5 sources, no change.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
@@ -1203,12 +1208,17 @@
           <t>Keep pmc.ncbi.nlm.nih.gov studies separate, reason stated; drop any study whose claim another listed source already covers.</t>
         </is>
       </c>
-      <c r="J10" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J10" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K10" s="5" t="inlineStr"/>
+      <c r="N10" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Reason confirmed: the repeated site hosts separate studies or papers, each with its own authors and year, each backing its own claim; 3 to 5 sources, no change.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
@@ -1377,12 +1387,17 @@
           <t>Keep pmc.ncbi.nlm.nih.gov studies separate, reason stated; drop any study whose claim another listed source already covers.</t>
         </is>
       </c>
-      <c r="J14" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J14" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K14" s="5" t="inlineStr"/>
+      <c r="N14" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Reason confirmed: the repeated site hosts separate studies or papers, each with its own authors and year, each backing its own claim; 3 to 5 sources, no change.</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
@@ -1551,12 +1566,17 @@
           <t>Keep pmc.ncbi.nlm.nih.gov studies separate, reason stated; drop any study whose claim another listed source already covers.</t>
         </is>
       </c>
-      <c r="J18" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J18" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K18" s="5" t="inlineStr"/>
+      <c r="N18" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Reason confirmed: the repeated site hosts separate studies or papers, each with its own authors and year, each backing its own claim; 3 to 5 sources, no change.</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
@@ -2356,12 +2376,17 @@
           <t>Combine fws.gov into one entry naming the pages unless each backs a distinct rule or listing.</t>
         </is>
       </c>
-      <c r="J37" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J37" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K37" s="5" t="inlineStr"/>
+      <c r="N37" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Combined: two USFWS fact sheets combined into one entry, 5 to 4.</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="5" t="inlineStr">
@@ -2403,12 +2428,17 @@
           <t>Keep sciencedirect.com studies separate, reason stated; drop any study whose claim another listed source already covers.</t>
         </is>
       </c>
-      <c r="J38" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J38" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K38" s="5" t="inlineStr"/>
+      <c r="N38" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Reason confirmed: the repeated site hosts separate studies or papers, each with its own authors and year, each backing its own claim; 3 to 5 sources, no change.</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="5" t="inlineStr">
@@ -2671,12 +2701,17 @@
           <t>Keep doi.org studies separate, reason stated; drop any study whose claim another listed source already covers.</t>
         </is>
       </c>
-      <c r="J44" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J44" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K44" s="5" t="inlineStr"/>
+      <c r="N44" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Reason confirmed: the repeated site hosts separate studies or papers, each with its own authors and year, each backing its own claim; 3 to 5 sources, no change.</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="5" t="inlineStr">
@@ -3928,12 +3963,17 @@
           <t>Keep doi.org studies separate, reason stated; drop any study whose claim another listed source already covers.</t>
         </is>
       </c>
-      <c r="J73" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J73" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K73" s="5" t="inlineStr"/>
+      <c r="N73" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Reason confirmed: the repeated site hosts separate studies or papers, each with its own authors and year, each backing its own claim; 3 to 5 sources, no change.</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="5" t="inlineStr">
@@ -5386,12 +5426,17 @@
           <t>Keep ncbi.nlm.nih.gov studies separate, reason stated; drop any study whose claim another listed source already covers.</t>
         </is>
       </c>
-      <c r="J109" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J109" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K109" s="5" t="inlineStr"/>
+      <c r="N109" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Reason confirmed: the repeated site hosts separate studies or papers, each with its own authors and year, each backing its own claim; 3 to 5 sources, no change.</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="5" t="inlineStr">
@@ -6620,12 +6665,17 @@
           <t>Keep sciencedirect.com studies separate, reason stated; drop any study whose claim another listed source already covers.</t>
         </is>
       </c>
-      <c r="J139" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J139" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K139" s="5" t="inlineStr"/>
+      <c r="N139" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Reason confirmed: the repeated site hosts separate studies or papers, each with its own authors and year, each backing its own claim; 3 to 5 sources, no change.</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="5" t="inlineStr">
@@ -7019,12 +7069,17 @@
           <t>Keep sciencedirect.com studies separate, reason stated; drop any study whose claim another listed source already covers.</t>
         </is>
       </c>
-      <c r="J148" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J148" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K148" s="5" t="inlineStr"/>
+      <c r="N148" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Reason confirmed: the repeated site hosts separate studies or papers, each with its own authors and year, each backing its own claim; 3 to 5 sources, no change.</t>
+        </is>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="5" t="inlineStr">
@@ -7366,12 +7421,17 @@
           <t>Keep pmc.ncbi.nlm.nih.gov studies separate, reason stated; drop any study whose claim another listed source already covers.</t>
         </is>
       </c>
-      <c r="J156" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J156" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K156" s="5" t="inlineStr"/>
+      <c r="N156" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Reason confirmed: the repeated site hosts separate studies or papers, each with its own authors and year, each backing its own claim; 3 to 5 sources, no change.</t>
+        </is>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="5" t="inlineStr">
@@ -8458,12 +8518,17 @@
           <t>Keep sciencedirect.com studies separate, reason stated; drop any study whose claim another listed source already covers.</t>
         </is>
       </c>
-      <c r="J185" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J185" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K185" s="5" t="inlineStr"/>
+      <c r="N185" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Reason confirmed: the repeated site hosts separate studies or papers, each with its own authors and year, each backing its own claim; 3 to 5 sources, no change.</t>
+        </is>
+      </c>
     </row>
     <row r="186">
       <c r="A186" s="5" t="inlineStr">
@@ -8649,14 +8714,19 @@
           <t>Keep pmc.ncbi.nlm.nih.gov studies separate, reason stated; drop any study whose claim another listed source already covers.</t>
         </is>
       </c>
-      <c r="J190" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J190" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K190" s="5" t="inlineStr">
         <is>
           <t>2026-10-06: same-site entries combined, 6 to 4 entries.</t>
+        </is>
+      </c>
+      <c r="N190" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Reason confirmed: the repeated site hosts separate studies or papers, each with its own authors and year, each backing its own claim; 3 to 5 sources, no change.</t>
         </is>
       </c>
     </row>
@@ -8845,12 +8915,17 @@
           <t>Keep doi.org studies separate, reason stated; drop any study whose claim another listed source already covers.</t>
         </is>
       </c>
-      <c r="J194" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J194" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K194" s="5" t="inlineStr"/>
+      <c r="N194" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Reason confirmed: the repeated site hosts separate studies or papers, each with its own authors and year, each backing its own claim; 3 to 5 sources, no change.</t>
+        </is>
+      </c>
     </row>
     <row r="195">
       <c r="A195" s="5" t="inlineStr">
@@ -8945,12 +9020,17 @@
           <t>Keep doi.org studies separate, reason stated; drop any study whose claim another listed source already covers.</t>
         </is>
       </c>
-      <c r="J196" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J196" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K196" s="5" t="inlineStr"/>
+      <c r="N196" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Reason confirmed: the repeated site hosts separate studies or papers, each with its own authors and year, each backing its own claim; 3 to 5 sources, no change.</t>
+        </is>
+      </c>
     </row>
     <row r="197">
       <c r="A197" s="5" t="inlineStr">
@@ -8992,12 +9072,17 @@
           <t>Keep pmc.ncbi.nlm.nih.gov studies separate, reason stated; drop any study whose claim another listed source already covers.</t>
         </is>
       </c>
-      <c r="J197" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J197" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K197" s="5" t="inlineStr"/>
+      <c r="N197" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Reason confirmed: the repeated site hosts separate studies or papers, each with its own authors and year, each backing its own claim; 3 to 5 sources, no change.</t>
+        </is>
+      </c>
     </row>
     <row r="198">
       <c r="A198" s="5" t="inlineStr">
@@ -9739,12 +9824,17 @@
           <t>Keep sciencedirect.com studies separate, reason stated; drop any study whose claim another listed source already covers.</t>
         </is>
       </c>
-      <c r="J216" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J216" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K216" s="5" t="inlineStr"/>
+      <c r="N216" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Reason confirmed: the repeated site hosts separate studies or papers, each with its own authors and year, each backing its own claim; 3 to 5 sources, no change.</t>
+        </is>
+      </c>
     </row>
     <row r="217">
       <c r="A217" s="5" t="inlineStr">
@@ -9942,12 +10032,17 @@
           <t>Keep doi.org studies separate, reason stated; drop any study whose claim another listed source already covers.</t>
         </is>
       </c>
-      <c r="J221" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J221" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K221" s="5" t="inlineStr"/>
+      <c r="N221" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Reason confirmed: the repeated site hosts separate studies or papers, each with its own authors and year, each backing its own claim; 3 to 5 sources, no change.</t>
+        </is>
+      </c>
     </row>
     <row r="222">
       <c r="A222" s="5" t="inlineStr">
@@ -10704,12 +10799,17 @@
           <t>Keep sciencedirect.com studies separate, reason stated; drop any study whose claim another listed source already covers.</t>
         </is>
       </c>
-      <c r="J240" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J240" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K240" s="5" t="inlineStr"/>
+      <c r="N240" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Reason confirmed: the repeated site hosts separate studies or papers, each with its own authors and year, each backing its own claim; 3 to 5 sources, no change.</t>
+        </is>
+      </c>
     </row>
     <row r="241">
       <c r="A241" s="5" t="inlineStr">
@@ -11038,12 +11138,17 @@
           <t>Keep pmc.ncbi.nlm.nih.gov studies separate, reason stated; drop any study whose claim another listed source already covers.</t>
         </is>
       </c>
-      <c r="J248" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J248" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K248" s="5" t="inlineStr"/>
+      <c r="N248" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Reason confirmed: the repeated site hosts separate studies or papers, each with its own authors and year, each backing its own claim; 3 to 5 sources, no change.</t>
+        </is>
+      </c>
     </row>
     <row r="249">
       <c r="A249" s="5" t="inlineStr">
@@ -12057,12 +12162,17 @@
           <t>Keep sciencedirect.com studies separate, reason stated; drop any study whose claim another listed source already covers.</t>
         </is>
       </c>
-      <c r="J274" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J274" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K274" s="5" t="inlineStr"/>
+      <c r="N274" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Reason confirmed: the repeated site hosts separate studies or papers, each with its own authors and year, each backing its own claim; 3 to 5 sources, no change.</t>
+        </is>
+      </c>
     </row>
     <row r="275">
       <c r="A275" s="5" t="inlineStr">
@@ -12431,12 +12541,17 @@
           <t>Keep doi.org studies separate, reason stated; drop any study whose claim another listed source already covers.</t>
         </is>
       </c>
-      <c r="J283" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J283" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K283" s="5" t="inlineStr"/>
+      <c r="N283" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Reason confirmed: the repeated site hosts separate studies or papers, each with its own authors and year, each backing its own claim; 3 to 5 sources, no change.</t>
+        </is>
+      </c>
     </row>
     <row r="284">
       <c r="A284" s="5" t="inlineStr">
@@ -13025,12 +13140,17 @@
           <t>Keep ncbi.nlm.nih.gov studies separate, reason stated; drop any study whose claim another listed source already covers.</t>
         </is>
       </c>
-      <c r="J298" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J298" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K298" s="5" t="inlineStr"/>
+      <c r="N298" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Reason confirmed: the repeated site hosts separate studies or papers, each with its own authors and year, each backing its own claim; 3 to 5 sources, no change.</t>
+        </is>
+      </c>
     </row>
     <row r="299">
       <c r="A299" s="5" t="inlineStr">
@@ -14176,14 +14296,19 @@
           <t>Combine usgs.gov into one entry naming the pages unless each backs a distinct rule or listing.</t>
         </is>
       </c>
-      <c r="J328" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J328" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K328" s="5" t="inlineStr">
         <is>
           <t>2026-10-06: same-site entries combined, 5 to 4 entries.</t>
+        </is>
+      </c>
+      <c r="N328" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Combined: three USGS Water Science School pages combined into one entry, 4 to 2; every claim keeps the same pages behind it.</t>
         </is>
       </c>
     </row>
@@ -14227,12 +14352,17 @@
           <t>Keep doi.org studies separate, reason stated; drop any study whose claim another listed source already covers.</t>
         </is>
       </c>
-      <c r="J329" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J329" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K329" s="5" t="inlineStr"/>
+      <c r="N329" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Reason confirmed: the repeated site hosts separate studies or papers, each with its own authors and year, each backing its own claim; 3 to 5 sources, no change.</t>
+        </is>
+      </c>
     </row>
     <row r="330">
       <c r="A330" s="5" t="inlineStr">
@@ -14313,14 +14443,19 @@
           <t>Keep sciencedirect.com studies separate, reason stated; drop any study whose claim another listed source already covers.</t>
         </is>
       </c>
-      <c r="J331" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J331" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K331" s="5" t="inlineStr">
         <is>
           <t>2026-10-06: same-site entries combined, 6 to 5 entries.</t>
+        </is>
+      </c>
+      <c r="N331" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Reason confirmed: the repeated site hosts separate studies or papers, each with its own authors and year, each backing its own claim; 3 to 5 sources, no change.</t>
         </is>
       </c>
     </row>
@@ -15501,12 +15636,17 @@
           <t>Keep doi.org studies separate, reason stated; drop any study whose claim another listed source already covers.</t>
         </is>
       </c>
-      <c r="J360" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J360" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K360" s="5" t="inlineStr"/>
+      <c r="N360" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Reason confirmed: the repeated site hosts separate studies or papers, each with its own authors and year, each backing its own claim; 3 to 5 sources, no change.</t>
+        </is>
+      </c>
     </row>
     <row r="361">
       <c r="A361" s="5" t="inlineStr">
@@ -16013,12 +16153,17 @@
           <t>Keep doi.org studies separate, reason stated; drop any study whose claim another listed source already covers.</t>
         </is>
       </c>
-      <c r="J373" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J373" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K373" s="5" t="inlineStr"/>
+      <c r="N373" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Reason confirmed: the repeated site hosts separate studies or papers, each with its own authors and year, each backing its own claim; 3 to 5 sources, no change.</t>
+        </is>
+      </c>
     </row>
     <row r="374">
       <c r="A374" s="5" t="inlineStr">
@@ -16204,12 +16349,17 @@
           <t>Keep cambridge.org studies separate, reason stated; drop any study whose claim another listed source already covers.</t>
         </is>
       </c>
-      <c r="J378" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J378" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K378" s="5" t="inlineStr"/>
+      <c r="N378" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Reason confirmed: the repeated site hosts separate studies or papers, each with its own authors and year, each backing its own claim; 3 to 5 sources, no change.</t>
+        </is>
+      </c>
     </row>
     <row r="379">
       <c r="A379" s="5" t="inlineStr">
@@ -16508,12 +16658,17 @@
           <t>Keep link.springer.com studies separate, reason stated; drop any study whose claim another listed source already covers.</t>
         </is>
       </c>
-      <c r="J385" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J385" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K385" s="5" t="inlineStr"/>
+      <c r="N385" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Reason confirmed: the repeated site hosts separate studies or papers, each with its own authors and year, each backing its own claim; 3 to 5 sources, no change.</t>
+        </is>
+      </c>
     </row>
     <row r="386">
       <c r="A386" s="5" t="inlineStr">
@@ -17515,12 +17670,17 @@
           <t>Keep pmc.ncbi.nlm.nih.gov studies separate, reason stated; drop any study whose claim another listed source already covers.</t>
         </is>
       </c>
-      <c r="J408" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J408" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K408" s="5" t="inlineStr"/>
+      <c r="N408" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Reason confirmed: the repeated site hosts separate studies or papers, each with its own authors and year, each backing its own claim; 3 to 5 sources, no change.</t>
+        </is>
+      </c>
     </row>
     <row r="409">
       <c r="A409" s="5" t="inlineStr">
@@ -18519,14 +18679,19 @@
           <t>Keep pmc.ncbi.nlm.nih.gov studies separate, reason stated; drop any study whose claim another listed source already covers.</t>
         </is>
       </c>
-      <c r="J433" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J433" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K433" s="5" t="inlineStr">
         <is>
           <t>2026-10-06: same-site entries combined, 6 to 5 entries.</t>
+        </is>
+      </c>
+      <c r="N433" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Reason confirmed: the repeated site hosts separate studies or papers, each with its own authors and year, each backing its own claim; 3 to 5 sources, no change.</t>
         </is>
       </c>
     </row>
@@ -18605,12 +18770,17 @@
           <t>Keep sciencedirect.com studies separate, reason stated; drop any study whose claim another listed source already covers.</t>
         </is>
       </c>
-      <c r="J435" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J435" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K435" s="5" t="inlineStr"/>
+      <c r="N435" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Reason confirmed: the repeated site hosts separate studies or papers, each with its own authors and year, each backing its own claim; 3 to 5 sources, no change.</t>
+        </is>
+      </c>
     </row>
     <row r="436">
       <c r="A436" s="5" t="inlineStr">
@@ -18916,12 +19086,17 @@
           <t>Keep doi.org studies separate, reason stated; drop any study whose claim another listed source already covers.</t>
         </is>
       </c>
-      <c r="J442" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J442" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K442" s="5" t="inlineStr"/>
+      <c r="N442" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Reason confirmed: the repeated site hosts separate studies or papers, each with its own authors and year, each backing its own claim; 3 to 5 sources, no change.</t>
+        </is>
+      </c>
     </row>
     <row r="443">
       <c r="A443" s="5" t="inlineStr">
@@ -19454,12 +19629,17 @@
           <t>Keep ncbi.nlm.nih.gov studies separate, reason stated; drop any study whose claim another listed source already covers.</t>
         </is>
       </c>
-      <c r="J454" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J454" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K454" s="5" t="inlineStr"/>
+      <c r="N454" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Reason confirmed: the repeated site hosts separate studies or papers, each with its own authors and year, each backing its own claim; 3 to 5 sources, no change.</t>
+        </is>
+      </c>
     </row>
     <row r="455">
       <c r="A455" s="5" t="inlineStr">
@@ -19592,12 +19772,17 @@
           <t>Keep sciencedirect.com studies separate, reason stated; drop any study whose claim another listed source already covers.</t>
         </is>
       </c>
-      <c r="J457" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J457" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K457" s="5" t="inlineStr"/>
+      <c r="N457" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Reason confirmed: the repeated site hosts separate studies or papers, each with its own authors and year, each backing its own claim; 3 to 5 sources, no change.</t>
+        </is>
+      </c>
     </row>
     <row r="458">
       <c r="A458" s="5" t="inlineStr">
@@ -19944,12 +20129,17 @@
           <t>Keep link.springer.com studies separate, reason stated; drop any study whose claim another listed source already covers.</t>
         </is>
       </c>
-      <c r="J465" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J465" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K465" s="5" t="inlineStr"/>
+      <c r="N465" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Reason confirmed: the repeated site hosts separate studies or papers, each with its own authors and year, each backing its own claim; 3 to 5 sources, no change.</t>
+        </is>
+      </c>
     </row>
     <row r="466">
       <c r="A466" s="5" t="inlineStr">
@@ -21278,12 +21468,17 @@
           <t>Keep doi.org studies separate, reason stated; drop any study whose claim another listed source already covers.</t>
         </is>
       </c>
-      <c r="J496" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J496" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K496" s="5" t="inlineStr"/>
+      <c r="N496" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Reason confirmed: the repeated site hosts separate studies or papers, each with its own authors and year, each backing its own claim; 3 to 5 sources, no change.</t>
+        </is>
+      </c>
     </row>
     <row r="497">
       <c r="A497" s="5" t="inlineStr">
@@ -21325,14 +21520,19 @@
           <t>Keep animallaw.info entries separate, reason stated.</t>
         </is>
       </c>
-      <c r="J497" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J497" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K497" s="5" t="inlineStr">
         <is>
           <t>2026-10-06: same-site entries combined, 5 to 4 entries.</t>
+        </is>
+      </c>
+      <c r="N497" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Combined: three Animal Legal &amp; Historical Center explainer pages (not statutes) combined, 4 to 2; every claim keeps the same pages behind it.</t>
         </is>
       </c>
     </row>
@@ -21673,12 +21873,17 @@
           <t>Keep ncbi.nlm.nih.gov studies separate, reason stated; drop any study whose claim another listed source already covers.</t>
         </is>
       </c>
-      <c r="J506" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J506" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K506" s="5" t="inlineStr"/>
+      <c r="N506" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Reason confirmed: the repeated site hosts separate studies or papers, each with its own authors and year, each backing its own claim; 3 to 5 sources, no change.</t>
+        </is>
+      </c>
     </row>
     <row r="507">
       <c r="A507" s="5" t="inlineStr">
@@ -21907,12 +22112,17 @@
           <t>Keep research-information.bris.ac.uk studies separate, reason stated; drop any study whose claim another listed source already covers.</t>
         </is>
       </c>
-      <c r="J512" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J512" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K512" s="5" t="inlineStr"/>
+      <c r="N512" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Reason confirmed: the repeated site hosts separate studies or papers, each with its own authors and year, each backing its own claim; 3 to 5 sources, no change.</t>
+        </is>
+      </c>
     </row>
     <row r="513">
       <c r="A513" s="5" t="inlineStr">
@@ -22602,12 +22812,17 @@
           <t>Keep sciencedirect.com studies separate, reason stated; drop any study whose claim another listed source already covers.</t>
         </is>
       </c>
-      <c r="J529" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J529" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K529" s="5" t="inlineStr"/>
+      <c r="N529" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Reason confirmed: the repeated site hosts separate studies or papers, each with its own authors and year, each backing its own claim; 3 to 5 sources, no change.</t>
+        </is>
+      </c>
     </row>
     <row r="530">
       <c r="A530" s="5" t="inlineStr">
@@ -22854,12 +23069,17 @@
           <t>Keep sciencedirect.com studies separate, reason stated; drop any study whose claim another listed source already covers.</t>
         </is>
       </c>
-      <c r="J535" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J535" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K535" s="5" t="inlineStr"/>
+      <c r="N535" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Reason confirmed: the repeated site hosts separate studies or papers, each with its own authors and year, each backing its own claim; 3 to 5 sources, no change.</t>
+        </is>
+      </c>
     </row>
     <row r="536">
       <c r="A536" s="5" t="inlineStr">
@@ -22901,12 +23121,17 @@
           <t>Keep jstage.jst.go.jp studies separate, reason stated; drop any study whose claim another listed source already covers.</t>
         </is>
       </c>
-      <c r="J536" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J536" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K536" s="5" t="inlineStr"/>
+      <c r="N536" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Reason confirmed: the repeated site hosts separate studies or papers, each with its own authors and year, each backing its own claim; 3 to 5 sources, no change.</t>
+        </is>
+      </c>
     </row>
     <row r="537">
       <c r="A537" s="5" t="inlineStr">
@@ -23191,12 +23416,17 @@
           <t>Keep sciencedirect.com studies separate, reason stated; drop any study whose claim another listed source already covers.</t>
         </is>
       </c>
-      <c r="J543" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J543" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K543" s="5" t="inlineStr"/>
+      <c r="N543" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Reason confirmed: the repeated site hosts separate studies or papers, each with its own authors and year, each backing its own claim; 3 to 5 sources, no change.</t>
+        </is>
+      </c>
     </row>
     <row r="544">
       <c r="A544" s="5" t="inlineStr">
@@ -23482,12 +23712,17 @@
           <t>Keep sciencedirect.com studies separate, reason stated; drop any study whose claim another listed source already covers.</t>
         </is>
       </c>
-      <c r="J550" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J550" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K550" s="5" t="inlineStr"/>
+      <c r="N550" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Reason confirmed: the repeated site hosts separate studies or papers, each with its own authors and year, each backing its own claim; 3 to 5 sources, no change.</t>
+        </is>
+      </c>
     </row>
     <row r="551">
       <c r="A551" s="5" t="inlineStr">
@@ -24353,12 +24588,17 @@
           <t>Combine antarctica.gov.au into one entry naming the pages unless each backs a distinct rule or listing.</t>
         </is>
       </c>
-      <c r="J570" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J570" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K570" s="5" t="inlineStr"/>
+      <c r="N570" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Combined: two Australian Antarctic Program pages combined, 4 to 3.</t>
+        </is>
+      </c>
     </row>
     <row r="571">
       <c r="A571" s="5" t="inlineStr">
@@ -24400,14 +24640,19 @@
           <t>Keep pmc.ncbi.nlm.nih.gov studies separate, reason stated; drop any study whose claim another listed source already covers.</t>
         </is>
       </c>
-      <c r="J571" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J571" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K571" s="5" t="inlineStr">
         <is>
           <t>2026-10-06: same-site entries combined, 6 to 5 entries.</t>
+        </is>
+      </c>
+      <c r="N571" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Reason confirmed: the repeated site hosts separate studies or papers, each with its own authors and year, each backing its own claim; 3 to 5 sources, no change.</t>
         </is>
       </c>
     </row>
@@ -24554,14 +24799,19 @@
           <t>Keep pmc.ncbi.nlm.nih.gov studies separate, reason stated; drop any study whose claim another listed source already covers.</t>
         </is>
       </c>
-      <c r="J574" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J574" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K574" s="5" t="inlineStr">
         <is>
           <t>2026-10-06: same-site entries combined, 6 to 5 entries.</t>
+        </is>
+      </c>
+      <c r="N574" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Reason confirmed: the repeated site hosts separate studies or papers, each with its own authors and year, each backing its own claim; 3 to 5 sources, no change.</t>
         </is>
       </c>
     </row>
@@ -25541,12 +25791,17 @@
           <t>Keep sciencedirect.com studies separate, reason stated; drop any study whose claim another listed source already covers.</t>
         </is>
       </c>
-      <c r="J599" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J599" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K599" s="5" t="inlineStr"/>
+      <c r="N599" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Reason confirmed: the repeated site hosts separate studies or papers, each with its own authors and year, each backing its own claim; 3 to 5 sources, no change.</t>
+        </is>
+      </c>
     </row>
     <row r="600">
       <c r="A600" s="5" t="inlineStr">
@@ -26164,12 +26419,17 @@
           <t>Keep sciencedirect.com studies separate, reason stated; drop any study whose claim another listed source already covers.</t>
         </is>
       </c>
-      <c r="J614" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J614" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K614" s="5" t="inlineStr"/>
+      <c r="N614" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Reason confirmed: the repeated site hosts separate studies or papers, each with its own authors and year, each backing its own claim; 3 to 5 sources, no change.</t>
+        </is>
+      </c>
     </row>
     <row r="615">
       <c r="A615" s="5" t="inlineStr">
@@ -28462,12 +28722,17 @@
           <t>Keep pmc.ncbi.nlm.nih.gov studies separate, reason stated; drop any study whose claim another listed source already covers.</t>
         </is>
       </c>
-      <c r="J671" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J671" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K671" s="5" t="inlineStr"/>
+      <c r="N671" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Reason confirmed: the repeated site hosts separate studies or papers, each with its own authors and year, each backing its own claim; 3 to 5 sources, no change.</t>
+        </is>
+      </c>
     </row>
     <row r="672">
       <c r="A672" s="5" t="inlineStr">
@@ -28681,12 +28946,17 @@
           <t>Combine aphis.usda.gov into one entry naming the pages unless each backs a distinct rule or listing.</t>
         </is>
       </c>
-      <c r="J676" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J676" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K676" s="5" t="inlineStr"/>
+      <c r="N676" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Combined: two APHIS pages combined, 5 to 4.</t>
+        </is>
+      </c>
     </row>
     <row r="677">
       <c r="A677" s="5" t="inlineStr">
@@ -29833,12 +30103,17 @@
           <t>Keep journals.plos.org studies separate, reason stated; drop any study whose claim another listed source already covers.</t>
         </is>
       </c>
-      <c r="J706" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J706" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K706" s="5" t="inlineStr"/>
+      <c r="N706" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Reason confirmed: the repeated site hosts separate studies or papers, each with its own authors and year, each backing its own claim; 3 to 5 sources, no change.</t>
+        </is>
+      </c>
     </row>
     <row r="707">
       <c r="A707" s="5" t="inlineStr">
@@ -30111,12 +30386,17 @@
           <t>Keep pmc.ncbi.nlm.nih.gov studies separate, reason stated; drop any study whose claim another listed source already covers.</t>
         </is>
       </c>
-      <c r="J713" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J713" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K713" s="5" t="inlineStr"/>
+      <c r="N713" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Reason confirmed: the repeated site hosts separate studies or papers, each with its own authors and year, each backing its own claim; 3 to 5 sources, no change.</t>
+        </is>
+      </c>
     </row>
     <row r="714">
       <c r="A714" s="5" t="inlineStr">
@@ -30298,12 +30578,17 @@
           <t>Keep pubmed.ncbi.nlm.nih.gov studies separate, reason stated; drop any study whose claim another listed source already covers.</t>
         </is>
       </c>
-      <c r="J717" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J717" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K717" s="5" t="inlineStr"/>
+      <c r="N717" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Reason confirmed: the repeated site hosts separate studies or papers, each with its own authors and year, each backing its own claim; 3 to 5 sources, no change.</t>
+        </is>
+      </c>
     </row>
     <row r="718">
       <c r="A718" s="5" t="inlineStr">
@@ -30672,14 +30957,19 @@
           <t>Keep sciencedirect.com studies separate, reason stated; drop any study whose claim another listed source already covers.</t>
         </is>
       </c>
-      <c r="J727" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J727" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K727" s="5" t="inlineStr">
         <is>
           <t>2026-10-06: same-site entries combined, 6 to 5 entries.</t>
+        </is>
+      </c>
+      <c r="N727" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Reason confirmed: the repeated site hosts separate studies or papers, each with its own authors and year, each backing its own claim; 3 to 5 sources, no change.</t>
         </is>
       </c>
     </row>
@@ -30963,14 +31253,19 @@
           <t>Keep pmc.ncbi.nlm.nih.gov studies separate, reason stated; drop any study whose claim another listed source already covers.</t>
         </is>
       </c>
-      <c r="J734" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J734" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K734" s="5" t="inlineStr">
         <is>
           <t>2026-10-06: same-site entries combined, 5 to 4 entries.</t>
+        </is>
+      </c>
+      <c r="N734" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Reason confirmed: the repeated site hosts separate studies or papers, each with its own authors and year, each backing its own claim; 3 to 5 sources, no change.</t>
         </is>
       </c>
     </row>
@@ -31162,12 +31457,17 @@
           <t>Keep sciencedirect.com studies separate, reason stated; drop any study whose claim another listed source already covers.</t>
         </is>
       </c>
-      <c r="J738" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J738" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K738" s="5" t="inlineStr"/>
+      <c r="N738" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Reason confirmed: the repeated site hosts separate studies or papers, each with its own authors and year, each backing its own claim; 3 to 5 sources, no change.</t>
+        </is>
+      </c>
     </row>
     <row r="739">
       <c r="A739" s="5" t="inlineStr">
@@ -31540,12 +31840,17 @@
           <t>Keep sciencedirect.com studies separate, reason stated; drop any study whose claim another listed source already covers.</t>
         </is>
       </c>
-      <c r="J747" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J747" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K747" s="5" t="inlineStr"/>
+      <c r="N747" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Reason confirmed: the repeated site hosts separate studies or papers, each with its own authors and year, each backing its own claim; 3 to 5 sources, no change.</t>
+        </is>
+      </c>
     </row>
     <row r="748">
       <c r="A748" s="5" t="inlineStr">
@@ -32201,12 +32506,17 @@
           <t>Keep doi.org studies separate, reason stated; drop any study whose claim another listed source already covers.</t>
         </is>
       </c>
-      <c r="J763" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J763" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K763" s="5" t="inlineStr"/>
+      <c r="N763" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Reason confirmed: the repeated site hosts separate studies or papers, each with its own authors and year, each backing its own claim; 3 to 5 sources, no change.</t>
+        </is>
+      </c>
     </row>
     <row r="764">
       <c r="A764" s="5" t="inlineStr">
@@ -32532,12 +32842,17 @@
           <t>Combine adfg.alaska.gov into one entry naming the pages unless each backs a distinct rule or listing.</t>
         </is>
       </c>
-      <c r="J771" s="6" t="inlineStr">
-        <is>
-          <t>Review</t>
+      <c r="J771" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K771" s="5" t="inlineStr"/>
+      <c r="N771" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06: Combined: two Alaska Department of Fish and Game pages combined, 5 to 4.</t>
+        </is>
+      </c>
     </row>
     <row r="772">
       <c r="A772" s="5" t="inlineStr">

</xml_diff>